<commit_message>
Suscripción (plan, vencimiento, WhatsApp), categorías adaptables a celular/tablet/web y función actualizar()
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbJcEhGkrHEGTN79GmSz3p
</commit_message>
<xml_diff>
--- a/docs/BaseDatos_Plantilla.xlsx
+++ b/docs/BaseDatos_Plantilla.xlsx
@@ -33,9 +33,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conocimiento" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertas" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suscripcion" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2026,7 +2027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:E199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7323,8 +7324,62 @@
         </is>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" s="5" t="inlineStr">
+        <is>
+          <t>Suscripcion</t>
+        </is>
+      </c>
+      <c r="B198" s="6" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="C198" s="6" t="inlineStr">
+        <is>
+          <t>Text (KEY)</t>
+        </is>
+      </c>
+      <c r="D198" s="6" t="inlineStr">
+        <is>
+          <t>Nombre del dato: Plan, Vencimiento o Contacto_WhatsApp</t>
+        </is>
+      </c>
+      <c r="E198" s="6" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="6" t="inlineStr">
+        <is>
+          <t>Suscripcion</t>
+        </is>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C199" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>Plan: lo que quieras (MENSUAL, ANUAL...). Vencimiento: fecha (dd-mm-aaaa); si queda vacío NO vence. Contacto_WhatsApp: número con código de país, sin + ni espacios</t>
+        </is>
+      </c>
+      <c r="E199" s="6" t="inlineStr">
+        <is>
+          <t>MENSUAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E197"/>
+  <autoFilter ref="A1:E199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8092,6 +8147,64 @@
       <formula1>"Crear,Editar,Eliminar,Exportar,Login"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Contacto_WhatsApp</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>56968005177</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Suscripción con servidor de licencias separado y bloqueo al vencer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbJcEhGkrHEGTN79GmSz3p
</commit_message>
<xml_diff>
--- a/docs/BaseDatos_Plantilla.xlsx
+++ b/docs/BaseDatos_Plantilla.xlsx
@@ -33,10 +33,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conocimiento" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertas" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suscripcion" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2027,7 +2026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E199"/>
+  <dimension ref="A1:E197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7324,62 +7323,8 @@
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="5" t="inlineStr">
-        <is>
-          <t>Suscripcion</t>
-        </is>
-      </c>
-      <c r="B198" s="6" t="inlineStr">
-        <is>
-          <t>Campo</t>
-        </is>
-      </c>
-      <c r="C198" s="6" t="inlineStr">
-        <is>
-          <t>Text (KEY)</t>
-        </is>
-      </c>
-      <c r="D198" s="6" t="inlineStr">
-        <is>
-          <t>Nombre del dato: Plan, Vencimiento o Contacto_WhatsApp</t>
-        </is>
-      </c>
-      <c r="E198" s="6" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="6" t="inlineStr">
-        <is>
-          <t>Suscripcion</t>
-        </is>
-      </c>
-      <c r="B199" s="6" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C199" s="6" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="D199" s="6" t="inlineStr">
-        <is>
-          <t>Plan: lo que quieras (MENSUAL, ANUAL...). Vencimiento: fecha (dd-mm-aaaa); si queda vacío NO vence. Contacto_WhatsApp: número con código de país, sin + ni espacios</t>
-        </is>
-      </c>
-      <c r="E199" s="6" t="inlineStr">
-        <is>
-          <t>MENSUAL</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E199"/>
+  <autoFilter ref="A1:E197"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8147,64 +8092,6 @@
       <formula1>"Crear,Editar,Eliminar,Exportar,Login"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Campo</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>Vencimiento</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Contacto_WhatsApp</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>56968005177</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Compras a proveedores, mapa en vivo de repartidores y APK con Capacitor
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbJcEhGkrHEGTN79GmSz3p
</commit_message>
<xml_diff>
--- a/docs/BaseDatos_Plantilla.xlsx
+++ b/docs/BaseDatos_Plantilla.xlsx
@@ -35,7 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$198</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1002,7 +1002,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Entrada compra,Salida venta,Ajuste,Merma,Anulacion venta"</formula1>
+      <formula1>"Entrada compra,Salida venta,Ajuste,Merma,Anulacion venta,Anulacion compra"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1362,7 +1362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1371,6 +1371,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1404,6 +1405,11 @@
           <t>Usuario</t>
         </is>
       </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1434,6 +1440,7 @@
           <t>master@minegocio.com</t>
         </is>
       </c>
+      <c r="G2" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2026,7 +2033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:E198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3599,7 +3606,7 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Enum: Entrada compra|Salida venta|Ajuste|Merma|Anulacion venta</t>
+          <t>Enum: Entrada compra|Salida venta|Ajuste|Merma|Anulacion venta|Anulacion compra</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
@@ -4636,56 +4643,52 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="inlineStr">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>Observación (N° de factura del proveedor, etc.)</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
         <is>
           <t>Detalle_Compra</t>
         </is>
       </c>
-      <c r="B98" s="6" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
         <is>
           <t>ID_DetCompra</t>
         </is>
       </c>
-      <c r="C98" s="6" t="inlineStr">
+      <c r="C99" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D98" s="6" t="inlineStr">
+      <c r="D99" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E98" s="6" t="inlineStr">
+      <c r="E99" s="6" t="inlineStr">
         <is>
           <t>DC0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="6" t="inlineStr">
-        <is>
-          <t>Detalle_Compra</t>
-        </is>
-      </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>ID_Compra</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Compras (Is a part of)</t>
-        </is>
-      </c>
-      <c r="D99" s="6" t="inlineStr">
-        <is>
-          <t>Compra a la que pertenece</t>
-        </is>
-      </c>
-      <c r="E99" s="6" t="inlineStr">
-        <is>
-          <t>CO0001</t>
         </is>
       </c>
     </row>
@@ -4697,22 +4700,22 @@
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>ID_Producto</t>
+          <t>ID_Compra</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Ref → Productos</t>
+          <t>Ref → Compras (Is a part of)</t>
         </is>
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>Producto</t>
+          <t>Compra a la que pertenece</t>
         </is>
       </c>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>CO0001</t>
         </is>
       </c>
     </row>
@@ -4724,22 +4727,22 @@
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>ID_Producto</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Ref → Productos</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Cantidad recibida</t>
+          <t>Producto</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
@@ -4751,22 +4754,22 @@
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>Costo_Unitario</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>Costo por unidad</t>
+          <t>Cantidad recibida</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -4778,76 +4781,76 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
+          <t>Costo_Unitario</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>Costo por unidad</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Detalle_Compra</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C103" s="6" t="inlineStr">
+      <c r="C104" s="6" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="D103" s="6" t="inlineStr">
+      <c r="D104" s="6" t="inlineStr">
         <is>
           <t>Cantidad × Costo (fórmula App formula)</t>
         </is>
       </c>
-      <c r="E103" s="6" t="inlineStr">
+      <c r="E104" s="6" t="inlineStr">
         <is>
           <t>43200</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="5" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
         <is>
           <t>Deliverys</t>
         </is>
       </c>
-      <c r="B104" s="6" t="inlineStr">
+      <c r="B105" s="6" t="inlineStr">
         <is>
           <t>ID_Delivery</t>
         </is>
       </c>
-      <c r="C104" s="6" t="inlineStr">
+      <c r="C105" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D104" s="6" t="inlineStr">
+      <c r="D105" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E104" s="6" t="inlineStr">
+      <c r="E105" s="6" t="inlineStr">
         <is>
           <t>D001</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="6" t="inlineStr">
-        <is>
-          <t>Deliverys</t>
-        </is>
-      </c>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="inlineStr">
-        <is>
-          <t>Text (LABEL)</t>
-        </is>
-      </c>
-      <c r="D105" s="6" t="inlineStr">
-        <is>
-          <t>Nombre del repartidor</t>
-        </is>
-      </c>
-      <c r="E105" s="6" t="inlineStr">
-        <is>
-          <t>Juan Pérez</t>
         </is>
       </c>
     </row>
@@ -4859,22 +4862,22 @@
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Telefono</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>Nombre del repartidor</t>
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
-          <t>+56944444444</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
     </row>
@@ -4886,22 +4889,22 @@
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Telefono</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Correo con el que entra a la app (perfil Delivery)</t>
+          <t>Teléfono</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>juan.delivery@correo.com</t>
+          <t>+56944444444</t>
         </is>
       </c>
     </row>
@@ -4913,22 +4916,22 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Vehiculo</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>Enum: Moto|Bicicleta|Auto|A pie</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
         <is>
-          <t>Medio de transporte</t>
+          <t>Correo con el que entra a la app (perfil Delivery)</t>
         </is>
       </c>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>Moto</t>
+          <t>juan.delivery@correo.com</t>
         </is>
       </c>
     </row>
@@ -4940,22 +4943,22 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Patente</t>
+          <t>Vehiculo</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Moto|Bicicleta|Auto|A pie</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Patente o placa</t>
+          <t>Medio de transporte</t>
         </is>
       </c>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>ABCD12</t>
+          <t>Moto</t>
         </is>
       </c>
     </row>
@@ -4967,22 +4970,22 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Patente</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>Enum: Disponible|Ocupado|Inactivo</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>Estado actual (cambia solo con automatización)</t>
+          <t>Patente o placa</t>
         </is>
       </c>
       <c r="E110" s="6" t="inlineStr">
         <is>
-          <t>Disponible</t>
+          <t>ABCD12</t>
         </is>
       </c>
     </row>
@@ -4994,22 +4997,22 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Tarifa_Base</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Enum: Disponible|Ocupado|Inactivo</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Tarifa base por servicio</t>
+          <t>Estado actual (cambia solo con automatización)</t>
         </is>
       </c>
       <c r="E111" s="6" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
@@ -5021,7 +5024,7 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Tarifa_Km</t>
+          <t>Tarifa_Base</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -5031,12 +5034,12 @@
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>Tarifa por km (opcional)</t>
+          <t>Tarifa base por servicio</t>
         </is>
       </c>
       <c r="E112" s="6" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1000</t>
         </is>
       </c>
     </row>
@@ -5048,22 +5051,22 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Tarifa_Km</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>Yes/No</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Tarifa por km (opcional)</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>300</t>
         </is>
       </c>
     </row>
@@ -5075,22 +5078,22 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Ultima_Ubicacion</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>Yes/No</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>Última posición reportada</t>
+          <t>Habilitado</t>
         </is>
       </c>
       <c r="E114" s="6" t="inlineStr">
         <is>
-          <t>-33.4500,-70.6600</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5102,76 +5105,76 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
+          <t>Ultima_Ubicacion</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>LatLong</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t>Última posición reportada</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>-33.4500,-70.6600</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>Deliverys</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
           <t>Fecha_Ubicacion</t>
         </is>
       </c>
-      <c r="C115" s="6" t="inlineStr">
+      <c r="C116" s="6" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr">
+      <c r="D116" s="6" t="inlineStr">
         <is>
           <t>Hora de la última posición</t>
         </is>
       </c>
-      <c r="E115" s="6" t="inlineStr">
+      <c r="E116" s="6" t="inlineStr">
         <is>
           <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="5" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
         <is>
           <t>Ventas</t>
         </is>
       </c>
-      <c r="B116" s="6" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>ID_Venta</t>
         </is>
       </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>Identificador. AppSheet: UNIQUEID() o correlativo</t>
         </is>
       </c>
-      <c r="E116" s="6" t="inlineStr">
+      <c r="E117" s="6" t="inlineStr">
         <is>
           <t>V000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="6" t="inlineStr">
-        <is>
-          <t>Ventas</t>
-        </is>
-      </c>
-      <c r="B117" s="6" t="inlineStr">
-        <is>
-          <t>Fecha_Hora</t>
-        </is>
-      </c>
-      <c r="C117" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D117" s="6" t="inlineStr">
-        <is>
-          <t>Automático: NOW()</t>
-        </is>
-      </c>
-      <c r="E117" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -5183,22 +5186,22 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>ID_Cliente</t>
+          <t>Fecha_Hora</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>Ref → Clientes</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>Cliente (se puede crear desde la venta con Add new)</t>
+          <t>Automático: NOW()</t>
         </is>
       </c>
       <c r="E118" s="6" t="inlineStr">
         <is>
-          <t>CL0001</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -5210,22 +5213,22 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>Tipo_Entrega</t>
+          <t>ID_Cliente</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>Enum: Retiro en local|Delivery</t>
+          <t>Ref → Clientes</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Si es Delivery se crea un servicio</t>
+          <t>Cliente (se puede crear desde la venta con Add new)</t>
         </is>
       </c>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>CL0001</t>
         </is>
       </c>
     </row>
@@ -5237,22 +5240,22 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Tipo_Entrega</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Enum: Retiro en local|Delivery</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>Suma de Detalle_Venta (virtual column)</t>
+          <t>Si es Delivery se crea un servicio</t>
         </is>
       </c>
       <c r="E120" s="6" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>Delivery</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5267,7 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Subtotal</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -5274,12 +5277,12 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Descuento total</t>
+          <t>Suma de Detalle_Venta (virtual column)</t>
         </is>
       </c>
       <c r="E121" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3000</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5294,7 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>Costo_Delivery</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -5301,12 +5304,12 @@
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>Monto del delivery (si aplica)</t>
+          <t>Descuento total</t>
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5321,7 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Costo_Delivery</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
@@ -5328,12 +5331,12 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Subtotal - Descuento + Costo_Delivery (virtual)</t>
+          <t>Monto del delivery (si aplica)</t>
         </is>
       </c>
       <c r="E123" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -5345,22 +5348,22 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>Metodo_Pago</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>Enum: Efectivo|Tarjeta|Transferencia|Mixto</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>Forma de pago</t>
+          <t>Subtotal - Descuento + Costo_Delivery (virtual)</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>4500</t>
         </is>
       </c>
     </row>
@@ -5372,22 +5375,22 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>Estado_Pago</t>
+          <t>Metodo_Pago</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Enum: Pagado|Pendiente|Parcial</t>
+          <t>Enum: Efectivo|Tarjeta|Transferencia|Mixto</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>Estado del pago</t>
+          <t>Forma de pago</t>
         </is>
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>Pagado</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
@@ -5399,22 +5402,22 @@
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Estado_Pago</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>Enum: Borrador|Confirmada|En despacho|Entregada|Anulada</t>
+          <t>Enum: Pagado|Pendiente|Parcial</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
         <is>
-          <t>Estado de la venta</t>
+          <t>Estado del pago</t>
         </is>
       </c>
       <c r="E126" s="6" t="inlineStr">
         <is>
-          <t>Confirmada</t>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -5426,22 +5429,22 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>Tipo_Documento</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Enum: Ticket|Boleta|Factura</t>
+          <t>Enum: Borrador|Confirmada|En despacho|Entregada|Anulada</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>Documento a emitir</t>
+          <t>Estado de la venta</t>
         </is>
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>Boleta</t>
+          <t>Confirmada</t>
         </is>
       </c>
     </row>
@@ -5453,22 +5456,22 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>Dia_Semana</t>
+          <t>Tipo_Documento</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Ticket|Boleta|Factura</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>Virtual/Apps Script: TEXT([Fecha_Hora],"dddd"). Sirve para KPI</t>
+          <t>Documento a emitir</t>
         </is>
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>Boleta</t>
         </is>
       </c>
     </row>
@@ -5480,76 +5483,76 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
+          <t>Dia_Semana</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>Virtual/Apps Script: TEXT([Fecha_Hora],"dddd"). Sirve para KPI</t>
+        </is>
+      </c>
+      <c r="E129" s="6" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
           <t>Usuario</t>
         </is>
       </c>
-      <c r="C129" s="6" t="inlineStr">
+      <c r="C130" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D129" s="6" t="inlineStr">
+      <c r="D130" s="6" t="inlineStr">
         <is>
           <t>Vendedor: USEREMAIL()</t>
         </is>
       </c>
-      <c r="E129" s="6" t="inlineStr">
+      <c r="E130" s="6" t="inlineStr">
         <is>
           <t>ventas@minegocio.com</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="5" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
         <is>
           <t>Detalle_Venta</t>
         </is>
       </c>
-      <c r="B130" s="6" t="inlineStr">
+      <c r="B131" s="6" t="inlineStr">
         <is>
           <t>ID_Detalle</t>
         </is>
       </c>
-      <c r="C130" s="6" t="inlineStr">
+      <c r="C131" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D130" s="6" t="inlineStr">
+      <c r="D131" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="E131" s="6" t="inlineStr">
         <is>
           <t>DV000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="6" t="inlineStr">
-        <is>
-          <t>Detalle_Venta</t>
-        </is>
-      </c>
-      <c r="B131" s="6" t="inlineStr">
-        <is>
-          <t>ID_Venta</t>
-        </is>
-      </c>
-      <c r="C131" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Ventas (Is a part of)</t>
-        </is>
-      </c>
-      <c r="D131" s="6" t="inlineStr">
-        <is>
-          <t>Venta a la que pertenece</t>
-        </is>
-      </c>
-      <c r="E131" s="6" t="inlineStr">
-        <is>
-          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -5561,22 +5564,22 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>ID_Producto</t>
+          <t>ID_Venta</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Ref → Productos</t>
+          <t>Ref → Ventas (Is a part of)</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>Producto vendido</t>
+          <t>Venta a la que pertenece</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -5588,22 +5591,22 @@
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>Nombre_Producto</t>
+          <t>ID_Producto</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Ref → Productos</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>Copia del nombre al momento de vender (historial fiel)</t>
+          <t>Producto vendido</t>
         </is>
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>Bebida cola 1.5L</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
@@ -5615,22 +5618,22 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>ID_Categoria</t>
+          <t>Nombre_Producto</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
         <is>
-          <t>Ref → Categorias</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>Copia de categoría para KPI por categoría</t>
+          <t>Copia del nombre al momento de vender (historial fiel)</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>Bebida cola 1.5L</t>
         </is>
       </c>
     </row>
@@ -5642,22 +5645,22 @@
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>ID_Categoria</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Ref → Categorias</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Cantidad vendida</t>
+          <t>Copia de categoría para KPI por categoría</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>C001</t>
         </is>
       </c>
     </row>
@@ -5669,22 +5672,22 @@
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>Precio_Unitario</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="C136" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>Precio al momento de la venta</t>
+          <t>Cantidad vendida</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5696,7 +5699,7 @@
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>Costo_Unitario</t>
+          <t>Precio_Unitario</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
@@ -5706,12 +5709,12 @@
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>Costo al momento de la venta (para margen)</t>
+          <t>Precio al momento de la venta</t>
         </is>
       </c>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5726,7 @@
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Costo_Unitario</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
@@ -5733,12 +5736,12 @@
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>Descuento de la línea</t>
+          <t>Costo al momento de la venta (para margen)</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>900</t>
         </is>
       </c>
     </row>
@@ -5750,7 +5753,7 @@
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -5760,12 +5763,12 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>Cantidad × Precio - Descuento</t>
+          <t>Descuento de la línea</t>
         </is>
       </c>
       <c r="E139" s="6" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5777,76 +5780,76 @@
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>Cantidad × Precio - Descuento</t>
+        </is>
+      </c>
+      <c r="E140" s="6" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>Detalle_Venta</t>
+        </is>
+      </c>
+      <c r="B141" s="6" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C140" s="6" t="inlineStr">
+      <c r="C141" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D140" s="6" t="inlineStr">
+      <c r="D141" s="6" t="inlineStr">
         <is>
           <t>Fecha de la venta (para filtros y KPI)</t>
         </is>
       </c>
-      <c r="E140" s="6" t="inlineStr">
+      <c r="E141" s="6" t="inlineStr">
         <is>
           <t>15-10-2026</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="5" t="inlineStr">
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
         <is>
           <t>Servicios_Delivery</t>
         </is>
       </c>
-      <c r="B141" s="6" t="inlineStr">
+      <c r="B142" s="6" t="inlineStr">
         <is>
           <t>ID_Servicio</t>
         </is>
       </c>
-      <c r="C141" s="6" t="inlineStr">
+      <c r="C142" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D141" s="6" t="inlineStr">
+      <c r="D142" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E141" s="6" t="inlineStr">
+      <c r="E142" s="6" t="inlineStr">
         <is>
           <t>S000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="6" t="inlineStr">
-        <is>
-          <t>Servicios_Delivery</t>
-        </is>
-      </c>
-      <c r="B142" s="6" t="inlineStr">
-        <is>
-          <t>ID_Venta</t>
-        </is>
-      </c>
-      <c r="C142" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Ventas</t>
-        </is>
-      </c>
-      <c r="D142" s="6" t="inlineStr">
-        <is>
-          <t>Venta asociada</t>
-        </is>
-      </c>
-      <c r="E142" s="6" t="inlineStr">
-        <is>
-          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -5858,22 +5861,22 @@
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>ID_Delivery</t>
+          <t>ID_Venta</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>Ref → Deliverys</t>
+          <t>Ref → Ventas</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Repartidor asignado</t>
+          <t>Venta asociada</t>
         </is>
       </c>
       <c r="E143" s="6" t="inlineStr">
         <is>
-          <t>D001</t>
+          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -5885,22 +5888,22 @@
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>Nombre_Delivery</t>
+          <t>ID_Delivery</t>
         </is>
       </c>
       <c r="C144" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Ref → Deliverys</t>
         </is>
       </c>
       <c r="D144" s="6" t="inlineStr">
         <is>
-          <t>Copia del nombre (historial fiel aunque cambie después)</t>
+          <t>Repartidor asignado</t>
         </is>
       </c>
       <c r="E144" s="6" t="inlineStr">
         <is>
-          <t>Juan Pérez</t>
+          <t>D001</t>
         </is>
       </c>
     </row>
@@ -5912,22 +5915,22 @@
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>Fecha_Asignacion</t>
+          <t>Nombre_Delivery</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>Automático: NOW() al asignar</t>
+          <t>Copia del nombre (historial fiel aunque cambie después)</t>
         </is>
       </c>
       <c r="E145" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
     </row>
@@ -5939,7 +5942,7 @@
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
-          <t>Fecha_Aceptado</t>
+          <t>Fecha_Asignacion</t>
         </is>
       </c>
       <c r="C146" s="6" t="inlineStr">
@@ -5949,10 +5952,14 @@
       </c>
       <c r="D146" s="6" t="inlineStr">
         <is>
-          <t>Se llena al presionar Aceptar</t>
-        </is>
-      </c>
-      <c r="E146" s="6" t="inlineStr"/>
+          <t>Automático: NOW() al asignar</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>15-10-2026 12:30</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
@@ -5962,7 +5969,7 @@
       </c>
       <c r="B147" s="6" t="inlineStr">
         <is>
-          <t>Fecha_Finalizado</t>
+          <t>Fecha_Aceptado</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
@@ -5972,7 +5979,7 @@
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Se llena al presionar Finalizar</t>
+          <t>Se llena al presionar Aceptar</t>
         </is>
       </c>
       <c r="E147" s="6" t="inlineStr"/>
@@ -5985,24 +5992,20 @@
       </c>
       <c r="B148" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Fecha_Finalizado</t>
         </is>
       </c>
       <c r="C148" s="6" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t>Solo la fecha, para filtrar por rango</t>
-        </is>
-      </c>
-      <c r="E148" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026</t>
-        </is>
-      </c>
+          <t>Se llena al presionar Finalizar</t>
+        </is>
+      </c>
+      <c r="E148" s="6" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
@@ -6012,22 +6015,22 @@
       </c>
       <c r="B149" s="6" t="inlineStr">
         <is>
-          <t>Direccion_Entrega</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Dirección de destino</t>
+          <t>Solo la fecha, para filtrar por rango</t>
         </is>
       </c>
       <c r="E149" s="6" t="inlineStr">
         <is>
-          <t>Av. Principal 123</t>
+          <t>15-10-2026</t>
         </is>
       </c>
     </row>
@@ -6039,22 +6042,22 @@
       </c>
       <c r="B150" s="6" t="inlineStr">
         <is>
-          <t>Destino_LatLong</t>
+          <t>Direccion_Entrega</t>
         </is>
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>Coordenadas destino</t>
+          <t>Dirección de destino</t>
         </is>
       </c>
       <c r="E150" s="6" t="inlineStr">
         <is>
-          <t>-33.4489,-70.6693</t>
+          <t>Av. Principal 123</t>
         </is>
       </c>
     </row>
@@ -6066,7 +6069,7 @@
       </c>
       <c r="B151" s="6" t="inlineStr">
         <is>
-          <t>Origen_LatLong</t>
+          <t>Destino_LatLong</t>
         </is>
       </c>
       <c r="C151" s="6" t="inlineStr">
@@ -6076,12 +6079,12 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Coordenadas del local</t>
+          <t>Coordenadas destino</t>
         </is>
       </c>
       <c r="E151" s="6" t="inlineStr">
         <is>
-          <t>-33.4372,-70.6506</t>
+          <t>-33.4489,-70.6693</t>
         </is>
       </c>
     </row>
@@ -6093,22 +6096,22 @@
       </c>
       <c r="B152" s="6" t="inlineStr">
         <is>
-          <t>Distancia_Km</t>
+          <t>Origen_LatLong</t>
         </is>
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>LatLong</t>
         </is>
       </c>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t>Km (manual o calculado con Apps Script/Maps)</t>
+          <t>Coordenadas del local</t>
         </is>
       </c>
       <c r="E152" s="6" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>-33.4372,-70.6506</t>
         </is>
       </c>
     </row>
@@ -6120,22 +6123,22 @@
       </c>
       <c r="B153" s="6" t="inlineStr">
         <is>
-          <t>Tiempo_Min</t>
+          <t>Distancia_Km</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Duración en minutos</t>
+          <t>Km (manual o calculado con Apps Script/Maps)</t>
         </is>
       </c>
       <c r="E153" s="6" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
@@ -6147,22 +6150,22 @@
       </c>
       <c r="B154" s="6" t="inlineStr">
         <is>
-          <t>Monto_Delivery</t>
+          <t>Tiempo_Min</t>
         </is>
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="D154" s="6" t="inlineStr">
         <is>
-          <t>Costo del servicio</t>
+          <t>Duración en minutos</t>
         </is>
       </c>
       <c r="E154" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -6174,22 +6177,22 @@
       </c>
       <c r="B155" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Monto_Delivery</t>
         </is>
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Enum: Asignado|Aceptado|En camino|Finalizado|Rechazado|Cancelado</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Estado del servicio</t>
+          <t>Costo del servicio</t>
         </is>
       </c>
       <c r="E155" s="6" t="inlineStr">
         <is>
-          <t>Asignado</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -6201,22 +6204,22 @@
       </c>
       <c r="B156" s="6" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>LongText</t>
+          <t>Enum: Asignado|Aceptado|En camino|Finalizado|Rechazado|Cancelado</t>
         </is>
       </c>
       <c r="D156" s="6" t="inlineStr">
         <is>
-          <t>Instrucciones para el repartidor</t>
+          <t>Estado del servicio</t>
         </is>
       </c>
       <c r="E156" s="6" t="inlineStr">
         <is>
-          <t>Llamar al llegar</t>
+          <t>Asignado</t>
         </is>
       </c>
     </row>
@@ -6228,76 +6231,76 @@
       </c>
       <c r="B157" s="6" t="inlineStr">
         <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="C157" s="6" t="inlineStr">
+        <is>
+          <t>LongText</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>Instrucciones para el repartidor</t>
+        </is>
+      </c>
+      <c r="E157" s="6" t="inlineStr">
+        <is>
+          <t>Llamar al llegar</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>Servicios_Delivery</t>
+        </is>
+      </c>
+      <c r="B158" s="6" t="inlineStr">
+        <is>
           <t>Usuario_Asigna</t>
         </is>
       </c>
-      <c r="C157" s="6" t="inlineStr">
+      <c r="C158" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D157" s="6" t="inlineStr">
+      <c r="D158" s="6" t="inlineStr">
         <is>
           <t>Quién asignó</t>
         </is>
       </c>
-      <c r="E157" s="6" t="inlineStr">
+      <c r="E158" s="6" t="inlineStr">
         <is>
           <t>ventas@minegocio.com</t>
         </is>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="5" t="inlineStr">
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
         <is>
           <t>Ubicaciones_Delivery</t>
         </is>
       </c>
-      <c r="B158" s="6" t="inlineStr">
+      <c r="B159" s="6" t="inlineStr">
         <is>
           <t>ID_Ubic</t>
         </is>
       </c>
-      <c r="C158" s="6" t="inlineStr">
+      <c r="C159" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D158" s="6" t="inlineStr">
+      <c r="D159" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E158" s="6" t="inlineStr">
+      <c r="E159" s="6" t="inlineStr">
         <is>
           <t>UB000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="6" t="inlineStr">
-        <is>
-          <t>Ubicaciones_Delivery</t>
-        </is>
-      </c>
-      <c r="B159" s="6" t="inlineStr">
-        <is>
-          <t>ID_Servicio</t>
-        </is>
-      </c>
-      <c r="C159" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Servicios_Delivery</t>
-        </is>
-      </c>
-      <c r="D159" s="6" t="inlineStr">
-        <is>
-          <t>Servicio en curso</t>
-        </is>
-      </c>
-      <c r="E159" s="6" t="inlineStr">
-        <is>
-          <t>S000001</t>
         </is>
       </c>
     </row>
@@ -6309,22 +6312,22 @@
       </c>
       <c r="B160" s="6" t="inlineStr">
         <is>
-          <t>ID_Delivery</t>
+          <t>ID_Servicio</t>
         </is>
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>Ref → Deliverys</t>
+          <t>Ref → Servicios_Delivery</t>
         </is>
       </c>
       <c r="D160" s="6" t="inlineStr">
         <is>
-          <t>Repartidor</t>
+          <t>Servicio en curso</t>
         </is>
       </c>
       <c r="E160" s="6" t="inlineStr">
         <is>
-          <t>D001</t>
+          <t>S000001</t>
         </is>
       </c>
     </row>
@@ -6336,22 +6339,22 @@
       </c>
       <c r="B161" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>ID_Delivery</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>Ref → Deliverys</t>
         </is>
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Posición registrada (AppSheet: HERE())</t>
+          <t>Repartidor</t>
         </is>
       </c>
       <c r="E161" s="6" t="inlineStr">
         <is>
-          <t>-33.4470,-70.6620</t>
+          <t>D001</t>
         </is>
       </c>
     </row>
@@ -6363,76 +6366,76 @@
       </c>
       <c r="B162" s="6" t="inlineStr">
         <is>
+          <t>LatLong</t>
+        </is>
+      </c>
+      <c r="C162" s="6" t="inlineStr">
+        <is>
+          <t>LatLong</t>
+        </is>
+      </c>
+      <c r="D162" s="6" t="inlineStr">
+        <is>
+          <t>Posición registrada (AppSheet: HERE())</t>
+        </is>
+      </c>
+      <c r="E162" s="6" t="inlineStr">
+        <is>
+          <t>-33.4470,-70.6620</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>Ubicaciones_Delivery</t>
+        </is>
+      </c>
+      <c r="B163" s="6" t="inlineStr">
+        <is>
           <t>Fecha_Hora</t>
         </is>
       </c>
-      <c r="C162" s="6" t="inlineStr">
+      <c r="C163" s="6" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D162" s="6" t="inlineStr">
+      <c r="D163" s="6" t="inlineStr">
         <is>
           <t>Momento del registro</t>
         </is>
       </c>
-      <c r="E162" s="6" t="inlineStr">
+      <c r="E163" s="6" t="inlineStr">
         <is>
           <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="5" t="inlineStr">
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
         <is>
           <t>Documentos</t>
         </is>
       </c>
-      <c r="B163" s="6" t="inlineStr">
+      <c r="B164" s="6" t="inlineStr">
         <is>
           <t>ID_Documento</t>
         </is>
       </c>
-      <c r="C163" s="6" t="inlineStr">
+      <c r="C164" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D163" s="6" t="inlineStr">
+      <c r="D164" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E163" s="6" t="inlineStr">
+      <c r="E164" s="6" t="inlineStr">
         <is>
           <t>DOC0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="6" t="inlineStr">
-        <is>
-          <t>Documentos</t>
-        </is>
-      </c>
-      <c r="B164" s="6" t="inlineStr">
-        <is>
-          <t>ID_Venta</t>
-        </is>
-      </c>
-      <c r="C164" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Ventas</t>
-        </is>
-      </c>
-      <c r="D164" s="6" t="inlineStr">
-        <is>
-          <t>Venta origen</t>
-        </is>
-      </c>
-      <c r="E164" s="6" t="inlineStr">
-        <is>
-          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -6444,22 +6447,22 @@
       </c>
       <c r="B165" s="6" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>ID_Venta</t>
         </is>
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Enum: Ticket|Boleta|Factura</t>
+          <t>Ref → Ventas</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Tipo de documento</t>
+          <t>Venta origen</t>
         </is>
       </c>
       <c r="E165" s="6" t="inlineStr">
         <is>
-          <t>Boleta</t>
+          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -6471,22 +6474,22 @@
       </c>
       <c r="B166" s="6" t="inlineStr">
         <is>
-          <t>Folio</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Ticket|Boleta|Factura</t>
         </is>
       </c>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t>Número correlativo interno (o folio SII si usas facturación electrónica)</t>
+          <t>Tipo de documento</t>
         </is>
       </c>
       <c r="E166" s="6" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>Boleta</t>
         </is>
       </c>
     </row>
@@ -6498,22 +6501,22 @@
       </c>
       <c r="B167" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Folio</t>
         </is>
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Emisión</t>
+          <t>Número correlativo interno (o folio SII si usas facturación electrónica)</t>
         </is>
       </c>
       <c r="E167" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>1001</t>
         </is>
       </c>
     </row>
@@ -6525,22 +6528,22 @@
       </c>
       <c r="B168" s="6" t="inlineStr">
         <is>
-          <t>Neto</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C168" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t>Monto neto</t>
+          <t>Emisión</t>
         </is>
       </c>
       <c r="E168" s="6" t="inlineStr">
         <is>
-          <t>3782</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6555,7 @@
       </c>
       <c r="B169" s="6" t="inlineStr">
         <is>
-          <t>Impuesto</t>
+          <t>Neto</t>
         </is>
       </c>
       <c r="C169" s="6" t="inlineStr">
@@ -6562,12 +6565,12 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>IVA u otro impuesto</t>
+          <t>Monto neto</t>
         </is>
       </c>
       <c r="E169" s="6" t="inlineStr">
         <is>
-          <t>718</t>
+          <t>3782</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6582,7 @@
       </c>
       <c r="B170" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Impuesto</t>
         </is>
       </c>
       <c r="C170" s="6" t="inlineStr">
@@ -6589,12 +6592,12 @@
       </c>
       <c r="D170" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>IVA u otro impuesto</t>
         </is>
       </c>
       <c r="E170" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>718</t>
         </is>
       </c>
     </row>
@@ -6606,22 +6609,22 @@
       </c>
       <c r="B171" s="6" t="inlineStr">
         <is>
-          <t>Formato</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
-          <t>Enum: Termica 58mm|Termica 80mm|A4 Carta</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Formato de impresión</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">
         <is>
-          <t>Termica 80mm</t>
+          <t>4500</t>
         </is>
       </c>
     </row>
@@ -6633,72 +6636,72 @@
       </c>
       <c r="B172" s="6" t="inlineStr">
         <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="C172" s="6" t="inlineStr">
+        <is>
+          <t>Enum: Termica 58mm|Termica 80mm|A4 Carta</t>
+        </is>
+      </c>
+      <c r="D172" s="6" t="inlineStr">
+        <is>
+          <t>Formato de impresión</t>
+        </is>
+      </c>
+      <c r="E172" s="6" t="inlineStr">
+        <is>
+          <t>Termica 80mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>Documentos</t>
+        </is>
+      </c>
+      <c r="B173" s="6" t="inlineStr">
+        <is>
           <t>PDF_URL</t>
         </is>
       </c>
-      <c r="C172" s="6" t="inlineStr">
+      <c r="C173" s="6" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="D172" s="6" t="inlineStr">
+      <c r="D173" s="6" t="inlineStr">
         <is>
           <t>PDF generado por Apps Script en Drive</t>
         </is>
       </c>
-      <c r="E172" s="6" t="inlineStr"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="5" t="inlineStr">
+      <c r="E173" s="6" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
         <is>
           <t>Categorias_Conocimiento</t>
         </is>
       </c>
-      <c r="B173" s="6" t="inlineStr">
+      <c r="B174" s="6" t="inlineStr">
         <is>
           <t>ID_CatCon</t>
         </is>
       </c>
-      <c r="C173" s="6" t="inlineStr">
+      <c r="C174" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D173" s="6" t="inlineStr">
+      <c r="D174" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E173" s="6" t="inlineStr">
+      <c r="E174" s="6" t="inlineStr">
         <is>
           <t>CK01</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="6" t="inlineStr">
-        <is>
-          <t>Categorias_Conocimiento</t>
-        </is>
-      </c>
-      <c r="B174" s="6" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C174" s="6" t="inlineStr">
-        <is>
-          <t>Text (LABEL)</t>
-        </is>
-      </c>
-      <c r="D174" s="6" t="inlineStr">
-        <is>
-          <t>Nombre de la categoría</t>
-        </is>
-      </c>
-      <c r="E174" s="6" t="inlineStr">
-        <is>
-          <t>Recetas</t>
         </is>
       </c>
     </row>
@@ -6710,76 +6713,76 @@
       </c>
       <c r="B175" s="6" t="inlineStr">
         <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="inlineStr">
+        <is>
+          <t>Text (LABEL)</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t>Nombre de la categoría</t>
+        </is>
+      </c>
+      <c r="E175" s="6" t="inlineStr">
+        <is>
+          <t>Recetas</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>Categorias_Conocimiento</t>
+        </is>
+      </c>
+      <c r="B176" s="6" t="inlineStr">
+        <is>
           <t>Imagen</t>
         </is>
       </c>
-      <c r="C175" s="6" t="inlineStr">
+      <c r="C176" s="6" t="inlineStr">
         <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="D175" s="6" t="inlineStr">
+      <c r="D176" s="6" t="inlineStr">
         <is>
           <t>Imagen opcional</t>
         </is>
       </c>
-      <c r="E175" s="6" t="inlineStr">
+      <c r="E176" s="6" t="inlineStr">
         <is>
           <t>Conocimiento_Images/recetas.png</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="5" t="inlineStr">
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
         <is>
           <t>Conocimiento</t>
         </is>
       </c>
-      <c r="B176" s="6" t="inlineStr">
+      <c r="B177" s="6" t="inlineStr">
         <is>
           <t>ID_Conocimiento</t>
         </is>
       </c>
-      <c r="C176" s="6" t="inlineStr">
+      <c r="C177" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D176" s="6" t="inlineStr">
+      <c r="D177" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E176" s="6" t="inlineStr">
+      <c r="E177" s="6" t="inlineStr">
         <is>
           <t>K0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="6" t="inlineStr">
-        <is>
-          <t>Conocimiento</t>
-        </is>
-      </c>
-      <c r="B177" s="6" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="C177" s="6" t="inlineStr">
-        <is>
-          <t>Text (LABEL)</t>
-        </is>
-      </c>
-      <c r="D177" s="6" t="inlineStr">
-        <is>
-          <t>Título del documento</t>
-        </is>
-      </c>
-      <c r="E177" s="6" t="inlineStr">
-        <is>
-          <t>Preparación salsa base</t>
         </is>
       </c>
     </row>
@@ -6791,22 +6794,22 @@
       </c>
       <c r="B178" s="6" t="inlineStr">
         <is>
-          <t>ID_CatCon</t>
+          <t>Titulo</t>
         </is>
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>Ref → Categorias_Conocimiento</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t>Categoría</t>
+          <t>Título del documento</t>
         </is>
       </c>
       <c r="E178" s="6" t="inlineStr">
         <is>
-          <t>CK01</t>
+          <t>Preparación salsa base</t>
         </is>
       </c>
     </row>
@@ -6818,22 +6821,22 @@
       </c>
       <c r="B179" s="6" t="inlineStr">
         <is>
-          <t>Archivo_PDF</t>
+          <t>ID_CatCon</t>
         </is>
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Ref → Categorias_Conocimiento</t>
         </is>
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>PDF subido (se guarda en Drive)</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="E179" s="6" t="inlineStr">
         <is>
-          <t>Conocimiento_Files/salsa_base.pdf</t>
+          <t>CK01</t>
         </is>
       </c>
     </row>
@@ -6845,22 +6848,22 @@
       </c>
       <c r="B180" s="6" t="inlineStr">
         <is>
-          <t>Descripcion</t>
+          <t>Archivo_PDF</t>
         </is>
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>LongText</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D180" s="6" t="inlineStr">
         <is>
-          <t>Resumen</t>
+          <t>PDF subido (se guarda en Drive)</t>
         </is>
       </c>
       <c r="E180" s="6" t="inlineStr">
         <is>
-          <t>Receta estándar de salsa base</t>
+          <t>Conocimiento_Files/salsa_base.pdf</t>
         </is>
       </c>
     </row>
@@ -6872,22 +6875,22 @@
       </c>
       <c r="B181" s="6" t="inlineStr">
         <is>
-          <t>Etiquetas</t>
+          <t>Descripcion</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>EnumList (Allow other values)</t>
+          <t>LongText</t>
         </is>
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>Etiquetas para buscar</t>
+          <t>Resumen</t>
         </is>
       </c>
       <c r="E181" s="6" t="inlineStr">
         <is>
-          <t>salsa, base</t>
+          <t>Receta estándar de salsa base</t>
         </is>
       </c>
     </row>
@@ -6899,22 +6902,22 @@
       </c>
       <c r="B182" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Etiquetas</t>
         </is>
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>EnumList (Allow other values)</t>
         </is>
       </c>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t>Automático</t>
+          <t>Etiquetas para buscar</t>
         </is>
       </c>
       <c r="E182" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>salsa, base</t>
         </is>
       </c>
     </row>
@@ -6926,76 +6929,76 @@
       </c>
       <c r="B183" s="6" t="inlineStr">
         <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C183" s="6" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="E183" s="6" t="inlineStr">
+        <is>
+          <t>15-10-2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="6" t="inlineStr">
+        <is>
+          <t>Conocimiento</t>
+        </is>
+      </c>
+      <c r="B184" s="6" t="inlineStr">
+        <is>
           <t>Usuario</t>
         </is>
       </c>
-      <c r="C183" s="6" t="inlineStr">
+      <c r="C184" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D183" s="6" t="inlineStr">
+      <c r="D184" s="6" t="inlineStr">
         <is>
           <t>Quién lo subió</t>
         </is>
       </c>
-      <c r="E183" s="6" t="inlineStr">
+      <c r="E184" s="6" t="inlineStr">
         <is>
           <t>master@minegocio.com</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="5" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
         <is>
           <t>Alertas</t>
         </is>
       </c>
-      <c r="B184" s="6" t="inlineStr">
+      <c r="B185" s="6" t="inlineStr">
         <is>
           <t>ID_Alerta</t>
         </is>
       </c>
-      <c r="C184" s="6" t="inlineStr">
+      <c r="C185" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D184" s="6" t="inlineStr">
+      <c r="D185" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E184" s="6" t="inlineStr">
+      <c r="E185" s="6" t="inlineStr">
         <is>
           <t>A000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="6" t="inlineStr">
-        <is>
-          <t>Alertas</t>
-        </is>
-      </c>
-      <c r="B185" s="6" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C185" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D185" s="6" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
-      <c r="E185" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -7007,22 +7010,22 @@
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>Enum: Stock minimo|Delivery finalizado|Delivery rechazado|Otro</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D186" s="6" t="inlineStr">
         <is>
-          <t>Tipo de alerta</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="E186" s="6" t="inlineStr">
         <is>
-          <t>Stock minimo</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -7034,22 +7037,22 @@
       </c>
       <c r="B187" s="6" t="inlineStr">
         <is>
-          <t>Referencia</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Stock minimo|Delivery finalizado|Delivery rechazado|Otro</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>ID_Producto o ID_Servicio</t>
+          <t>Tipo de alerta</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>Stock minimo</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7064,7 @@
       </c>
       <c r="B188" s="6" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="C188" s="6" t="inlineStr">
@@ -7071,12 +7074,12 @@
       </c>
       <c r="D188" s="6" t="inlineStr">
         <is>
-          <t>Texto de la alerta</t>
+          <t>ID_Producto o ID_Servicio</t>
         </is>
       </c>
       <c r="E188" s="6" t="inlineStr">
         <is>
-          <t>Bebida cola 1.5L llegó al stock mínimo (10)</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
@@ -7088,22 +7091,22 @@
       </c>
       <c r="B189" s="6" t="inlineStr">
         <is>
-          <t>Para_Rol</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>Ref → Roles</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Rol que debe verla</t>
+          <t>Texto de la alerta</t>
         </is>
       </c>
       <c r="E189" s="6" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>Bebida cola 1.5L llegó al stock mínimo (10)</t>
         </is>
       </c>
     </row>
@@ -7115,76 +7118,76 @@
       </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
+          <t>Para_Rol</t>
+        </is>
+      </c>
+      <c r="C190" s="6" t="inlineStr">
+        <is>
+          <t>Ref → Roles</t>
+        </is>
+      </c>
+      <c r="D190" s="6" t="inlineStr">
+        <is>
+          <t>Rol que debe verla</t>
+        </is>
+      </c>
+      <c r="E190" s="6" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="6" t="inlineStr">
+        <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="B191" s="6" t="inlineStr">
+        <is>
           <t>Leida</t>
         </is>
       </c>
-      <c r="C190" s="6" t="inlineStr">
+      <c r="C191" s="6" t="inlineStr">
         <is>
           <t>Yes/No</t>
         </is>
       </c>
-      <c r="D190" s="6" t="inlineStr">
+      <c r="D191" s="6" t="inlineStr">
         <is>
           <t>Marcada como leída</t>
         </is>
       </c>
-      <c r="E190" s="6" t="inlineStr">
+      <c r="E191" s="6" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="5" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="5" t="inlineStr">
         <is>
           <t>Auditoria</t>
         </is>
       </c>
-      <c r="B191" s="6" t="inlineStr">
+      <c r="B192" s="6" t="inlineStr">
         <is>
           <t>ID_Log</t>
         </is>
       </c>
-      <c r="C191" s="6" t="inlineStr">
+      <c r="C192" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D191" s="6" t="inlineStr">
+      <c r="D192" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E191" s="6" t="inlineStr">
+      <c r="E192" s="6" t="inlineStr">
         <is>
           <t>L000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="6" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="B192" s="6" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C192" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D192" s="6" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
-      <c r="E192" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -7196,22 +7199,22 @@
       </c>
       <c r="B193" s="6" t="inlineStr">
         <is>
-          <t>Usuario</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Quién</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="E193" s="6" t="inlineStr">
         <is>
-          <t>master@minegocio.com</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -7223,22 +7226,22 @@
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t>Modulo</t>
+          <t>Usuario</t>
         </is>
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D194" s="6" t="inlineStr">
         <is>
-          <t>Módulo afectado</t>
+          <t>Quién</t>
         </is>
       </c>
       <c r="E194" s="6" t="inlineStr">
         <is>
-          <t>Inventario</t>
+          <t>master@minegocio.com</t>
         </is>
       </c>
     </row>
@@ -7250,22 +7253,22 @@
       </c>
       <c r="B195" s="6" t="inlineStr">
         <is>
-          <t>Accion</t>
+          <t>Modulo</t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
         <is>
-          <t>Enum: Crear|Editar|Eliminar|Exportar|Login</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Qué hizo</t>
+          <t>Módulo afectado</t>
         </is>
       </c>
       <c r="E195" s="6" t="inlineStr">
         <is>
-          <t>Crear</t>
+          <t>Inventario</t>
         </is>
       </c>
     </row>
@@ -7277,22 +7280,22 @@
       </c>
       <c r="B196" s="6" t="inlineStr">
         <is>
-          <t>Registro</t>
+          <t>Accion</t>
         </is>
       </c>
       <c r="C196" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Crear|Editar|Eliminar|Exportar|Login</t>
         </is>
       </c>
       <c r="D196" s="6" t="inlineStr">
         <is>
-          <t>ID del registro afectado</t>
+          <t>Qué hizo</t>
         </is>
       </c>
       <c r="E196" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>Crear</t>
         </is>
       </c>
     </row>
@@ -7304,27 +7307,54 @@
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
+          <t>Registro</t>
+        </is>
+      </c>
+      <c r="C197" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D197" s="6" t="inlineStr">
+        <is>
+          <t>ID del registro afectado</t>
+        </is>
+      </c>
+      <c r="E197" s="6" t="inlineStr">
+        <is>
+          <t>P0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="6" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="B198" s="6" t="inlineStr">
+        <is>
           <t>Detalle</t>
         </is>
       </c>
-      <c r="C197" s="6" t="inlineStr">
+      <c r="C198" s="6" t="inlineStr">
         <is>
           <t>LongText</t>
         </is>
       </c>
-      <c r="D197" s="6" t="inlineStr">
+      <c r="D198" s="6" t="inlineStr">
         <is>
           <t>Detalle del cambio</t>
         </is>
       </c>
-      <c r="E197" s="6" t="inlineStr">
+      <c r="E198" s="6" t="inlineStr">
         <is>
           <t>Producto creado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E197"/>
+  <autoFilter ref="A1:E198"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Venta 'Para servir' e ícono propio por negocio para la APK
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbJcEhGkrHEGTN79GmSz3p
</commit_message>
<xml_diff>
--- a/docs/BaseDatos_Plantilla.xlsx
+++ b/docs/BaseDatos_Plantilla.xlsx
@@ -1869,7 +1869,7 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Retiro en local,Delivery"</formula1>
+      <formula1>"Retiro en local,Para servir,Delivery"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Efectivo,Tarjeta,Transferencia,Mixto"</formula1>
@@ -5245,7 +5245,7 @@
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Enum: Retiro en local|Delivery</t>
+          <t>Enum: Retiro en local|Para servir|Delivery</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Comanda de cocina: referencia, notas por producto, pestaña e impresión separada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbJcEhGkrHEGTN79GmSz3p
</commit_message>
<xml_diff>
--- a/docs/BaseDatos_Plantilla.xlsx
+++ b/docs/BaseDatos_Plantilla.xlsx
@@ -35,7 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DICCIONARIO'!$A$1:$E$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -726,6 +726,7 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -799,6 +800,11 @@
           <t>Fecha_Creacion</t>
         </is>
       </c>
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>Va_A_Cocina</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -869,10 +875,18 @@
       <c r="N2" s="11" t="n">
         <v>46310.52083333334</v>
       </c>
+      <c r="O2" s="10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1705,7 +1719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1722,6 +1736,8 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1795,6 +1811,16 @@
           <t>Usuario</t>
         </is>
       </c>
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>Referencia</t>
+        </is>
+      </c>
+      <c r="P1" s="8" t="inlineStr">
+        <is>
+          <t>Nota_Cocina</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1863,6 +1889,16 @@
       <c r="N2" s="10" t="inlineStr">
         <is>
           <t>ventas@minegocio.com</t>
+        </is>
+      </c>
+      <c r="O2" s="10" t="inlineStr">
+        <is>
+          <t>Mesa 4</t>
+        </is>
+      </c>
+      <c r="P2" s="10" t="inlineStr">
+        <is>
+          <t>Todo para llevar junto</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1944,8 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1966,6 +2004,16 @@
           <t>Fecha</t>
         </is>
       </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>Va_A_Cocina</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -2021,8 +2069,19 @@
       <c r="K2" s="12" t="n">
         <v>46310</v>
       </c>
+      <c r="L2" s="10" t="inlineStr"/>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2033,7 +2092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E198"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3513,56 +3572,56 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Va_A_Cocina</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Yes/No</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Si es TRUE (o vacío) el producto sale en la comanda de cocina</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Movimientos_Inventario</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>ID_Mov</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>M00001</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>Movimientos_Inventario</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -3574,22 +3633,22 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>ID_Producto</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Ref → Productos</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Producto afectado</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -3601,22 +3660,22 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>ID_Producto</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Enum: Entrada compra|Salida venta|Ajuste|Merma|Anulacion venta|Anulacion compra</t>
+          <t>Ref → Productos</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Motivo del movimiento</t>
+          <t>Producto afectado</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Salida venta</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
@@ -3628,22 +3687,22 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Enum: Entrada compra|Salida venta|Ajuste|Merma|Anulacion venta|Anulacion compra</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Positiva siempre; el Tipo define si suma o resta</t>
+          <t>Motivo del movimiento</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Salida venta</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3714,7 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Stock_Antes</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3665,12 +3724,12 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Stock antes del movimiento</t>
+          <t>Positiva siempre; el Tipo define si suma o resta</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3741,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Stock_Despues</t>
+          <t>Stock_Antes</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -3692,12 +3751,12 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Stock luego del movimiento</t>
+          <t>Stock antes del movimiento</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>50</t>
         </is>
       </c>
     </row>
@@ -3709,22 +3768,22 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Referencia</t>
+          <t>Stock_Despues</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>ID_Venta o ID_Compra que lo originó</t>
+          <t>Stock luego del movimiento</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>V000001</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -3736,22 +3795,22 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Usuario</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Quién lo hizo: USEREMAIL()</t>
+          <t>ID_Venta o ID_Compra que lo originó</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>master@minegocio.com</t>
+          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -3763,72 +3822,72 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
+          <t>Usuario</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Quién lo hizo: USEREMAIL()</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>master@minegocio.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Movimientos_Inventario</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
+      <c r="D66" s="6" t="inlineStr">
         <is>
           <t>Observación</t>
         </is>
       </c>
-      <c r="E65" s="6" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="E66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>Clientes</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>ID_Cliente</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="E67" s="6" t="inlineStr">
         <is>
           <t>CL0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr">
-        <is>
-          <t>Clientes</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr">
-        <is>
-          <t>Text (LABEL)</t>
-        </is>
-      </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Nombre o razón social</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr">
-        <is>
-          <t>María González</t>
         </is>
       </c>
     </row>
@@ -3840,22 +3899,22 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Documento</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>RUT / DNI / RIF</t>
+          <t>Nombre o razón social</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>12.345.678-9</t>
+          <t>María González</t>
         </is>
       </c>
     </row>
@@ -3867,22 +3926,22 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Telefono</t>
+          <t>Documento</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>RUT / DNI / RIF</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>+56922222222</t>
+          <t>12.345.678-9</t>
         </is>
       </c>
     </row>
@@ -3894,22 +3953,22 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Telefono</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>Correo (para enviar boletas/facturas)</t>
+          <t>Teléfono</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>maria@correo.com</t>
+          <t>+56922222222</t>
         </is>
       </c>
     </row>
@@ -3921,22 +3980,22 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Direccion</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Dirección principal</t>
+          <t>Correo (para enviar boletas/facturas)</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Av. Principal 123</t>
+          <t>maria@correo.com</t>
         </is>
       </c>
     </row>
@@ -3948,22 +4007,22 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Ubicacion</t>
+          <t>Direccion</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Coordenadas para el mapa</t>
+          <t>Dirección principal</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>-33.4489,-70.6693</t>
+          <t>Av. Principal 123</t>
         </is>
       </c>
     </row>
@@ -3975,22 +4034,22 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Ubicacion</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>LongText</t>
+          <t>LatLong</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Observaciones</t>
+          <t>Coordenadas para el mapa</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Prefiere entrega en la tarde</t>
+          <t>-33.4489,-70.6693</t>
         </is>
       </c>
     </row>
@@ -4002,76 +4061,76 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>LongText</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>Prefiere entrega en la tarde</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Clientes</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
           <t>Fecha_Creacion</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="D75" s="6" t="inlineStr">
         <is>
           <t>Automático</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="E75" s="6" t="inlineStr">
         <is>
           <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>Proveedores</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>ID_Proveedor</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C76" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="D76" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E75" s="6" t="inlineStr">
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>PR001</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>Proveedores</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C76" s="6" t="inlineStr">
-        <is>
-          <t>Text (LABEL)</t>
-        </is>
-      </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Empresa o persona</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
-        <is>
-          <t>Distribuidora Norte</t>
         </is>
       </c>
     </row>
@@ -4083,22 +4142,22 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Documento</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>RUT / ID fiscal</t>
+          <t>Empresa o persona</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>76.111.222-3</t>
+          <t>Distribuidora Norte</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4169,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Contacto</t>
+          <t>Documento</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4120,12 +4179,12 @@
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Persona de contacto</t>
+          <t>RUT / ID fiscal</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Carlos Soto</t>
+          <t>76.111.222-3</t>
         </is>
       </c>
     </row>
@@ -4137,22 +4196,22 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Telefono</t>
+          <t>Contacto</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>Persona de contacto</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>+56933333333</t>
+          <t>Carlos Soto</t>
         </is>
       </c>
     </row>
@@ -4164,22 +4223,22 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Telefono</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Correo</t>
+          <t>Teléfono</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>ventas@distnorte.com</t>
+          <t>+56933333333</t>
         </is>
       </c>
     </row>
@@ -4191,22 +4250,22 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Direccion</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Dirección</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Calle Industrial 45</t>
+          <t>ventas@distnorte.com</t>
         </is>
       </c>
     </row>
@@ -4218,22 +4277,22 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Dias_Visita</t>
+          <t>Direccion</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>EnumList: Lunes|Martes|Miercoles|Jueves|Viernes|Sabado|Domingo</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>Días en que visita tu local</t>
+          <t>Dirección</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Martes, Viernes</t>
+          <t>Calle Industrial 45</t>
         </is>
       </c>
     </row>
@@ -4245,22 +4304,22 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Ultima_Visita</t>
+          <t>Dias_Visita</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>EnumList: Lunes|Martes|Miercoles|Jueves|Viernes|Sabado|Domingo</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Última visita registrada</t>
+          <t>Días en que visita tu local</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>Martes, Viernes</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4331,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Proxima_Visita</t>
+          <t>Ultima_Visita</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -4282,12 +4341,12 @@
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>Próxima visita estimada</t>
+          <t>Última visita registrada</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -4299,76 +4358,76 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
+          <t>Proxima_Visita</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>Próxima visita estimada</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>Proveedores</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="C85" s="6" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>LongText</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>Condiciones, plazos, etc.</t>
         </is>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Pago a 15 días</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
         <is>
           <t>Visitas_Proveedor</t>
         </is>
       </c>
-      <c r="B86" s="6" t="inlineStr">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>ID_Visita</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="E87" s="6" t="inlineStr">
         <is>
           <t>VP0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>Visitas_Proveedor</t>
-        </is>
-      </c>
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>ID_Proveedor</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Proveedores</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>Proveedor</t>
-        </is>
-      </c>
-      <c r="E87" s="6" t="inlineStr">
-        <is>
-          <t>PR001</t>
         </is>
       </c>
     </row>
@@ -4380,22 +4439,22 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>ID_Proveedor</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Ref → Proveedores</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>Fecha de la visita</t>
+          <t>Proveedor</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>13-10-2026</t>
+          <t>PR001</t>
         </is>
       </c>
     </row>
@@ -4407,22 +4466,22 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Enum: Proveedor visita el local|Yo voy al proveedor</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Quién se desplaza</t>
+          <t>Fecha de la visita</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Proveedor visita el local</t>
+          <t>13-10-2026</t>
         </is>
       </c>
     </row>
@@ -4434,22 +4493,22 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>LongText</t>
+          <t>Enum: Proveedor visita el local|Yo voy al proveedor</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>Detalle (qué se pidió, qué se pagó)</t>
+          <t>Quién se desplaza</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Pedido semanal</t>
+          <t>Proveedor visita el local</t>
         </is>
       </c>
     </row>
@@ -4461,76 +4520,76 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>LongText</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>Detalle (qué se pidió, qué se pagó)</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Pedido semanal</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>Visitas_Proveedor</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
           <t>Usuario</t>
         </is>
       </c>
-      <c r="C91" s="6" t="inlineStr">
+      <c r="C92" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D91" s="6" t="inlineStr">
+      <c r="D92" s="6" t="inlineStr">
         <is>
           <t>Quién lo registró</t>
         </is>
       </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="E92" s="6" t="inlineStr">
         <is>
           <t>master@minegocio.com</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="5" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
         <is>
           <t>Compras</t>
         </is>
       </c>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>ID_Compra</t>
         </is>
       </c>
-      <c r="C92" s="6" t="inlineStr">
+      <c r="C93" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr">
+      <c r="D93" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E92" s="6" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>CO0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D93" s="6" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -4542,22 +4601,22 @@
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>ID_Proveedor</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Ref → Proveedores</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>Proveedor</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>PR001</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -4569,22 +4628,22 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>ID_Proveedor</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Ref → Proveedores</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Suma de Detalle_Compra (virtual column en AppSheet)</t>
+          <t>Proveedor</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>43200</t>
+          <t>PR001</t>
         </is>
       </c>
     </row>
@@ -4596,22 +4655,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Enum: Pendiente|Recibida|Anulada</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>Al pasar a Recibida suma stock</t>
+          <t>Suma de Detalle_Compra (virtual column en AppSheet)</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>Recibida</t>
+          <t>43200</t>
         </is>
       </c>
     </row>
@@ -4623,22 +4682,22 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>Usuario</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Enum: Pendiente|Recibida|Anulada</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Quién registró</t>
+          <t>Al pasar a Recibida suma stock</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>master@minegocio.com</t>
+          <t>Recibida</t>
         </is>
       </c>
     </row>
@@ -4650,72 +4709,72 @@
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
+          <t>Usuario</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>Quién registró</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>master@minegocio.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="C98" s="6" t="inlineStr">
+      <c r="C99" s="6" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="D98" s="6" t="inlineStr">
+      <c r="D99" s="6" t="inlineStr">
         <is>
           <t>Observación (N° de factura del proveedor, etc.)</t>
         </is>
       </c>
-      <c r="E98" s="6" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="5" t="inlineStr">
+      <c r="E99" s="6" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
         <is>
           <t>Detalle_Compra</t>
         </is>
       </c>
-      <c r="B99" s="6" t="inlineStr">
+      <c r="B100" s="6" t="inlineStr">
         <is>
           <t>ID_DetCompra</t>
         </is>
       </c>
-      <c r="C99" s="6" t="inlineStr">
+      <c r="C100" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D99" s="6" t="inlineStr">
+      <c r="D100" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E99" s="6" t="inlineStr">
+      <c r="E100" s="6" t="inlineStr">
         <is>
           <t>DC0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="6" t="inlineStr">
-        <is>
-          <t>Detalle_Compra</t>
-        </is>
-      </c>
-      <c r="B100" s="6" t="inlineStr">
-        <is>
-          <t>ID_Compra</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Compras (Is a part of)</t>
-        </is>
-      </c>
-      <c r="D100" s="6" t="inlineStr">
-        <is>
-          <t>Compra a la que pertenece</t>
-        </is>
-      </c>
-      <c r="E100" s="6" t="inlineStr">
-        <is>
-          <t>CO0001</t>
         </is>
       </c>
     </row>
@@ -4727,22 +4786,22 @@
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>ID_Producto</t>
+          <t>ID_Compra</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Ref → Productos</t>
+          <t>Ref → Compras (Is a part of)</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Producto</t>
+          <t>Compra a la que pertenece</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>CO0001</t>
         </is>
       </c>
     </row>
@@ -4754,22 +4813,22 @@
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>ID_Producto</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Ref → Productos</t>
         </is>
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>Cantidad recibida</t>
+          <t>Producto</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
@@ -4781,22 +4840,22 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>Costo_Unitario</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Costo por unidad</t>
+          <t>Cantidad recibida</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -4808,76 +4867,76 @@
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
+          <t>Costo_Unitario</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="inlineStr">
+        <is>
+          <t>Costo por unidad</t>
+        </is>
+      </c>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>Detalle_Compra</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C104" s="6" t="inlineStr">
+      <c r="C105" s="6" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="D104" s="6" t="inlineStr">
+      <c r="D105" s="6" t="inlineStr">
         <is>
           <t>Cantidad × Costo (fórmula App formula)</t>
         </is>
       </c>
-      <c r="E104" s="6" t="inlineStr">
+      <c r="E105" s="6" t="inlineStr">
         <is>
           <t>43200</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t>Deliverys</t>
         </is>
       </c>
-      <c r="B105" s="6" t="inlineStr">
+      <c r="B106" s="6" t="inlineStr">
         <is>
           <t>ID_Delivery</t>
         </is>
       </c>
-      <c r="C105" s="6" t="inlineStr">
+      <c r="C106" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D105" s="6" t="inlineStr">
+      <c r="D106" s="6" t="inlineStr">
         <is>
           <t>Identificador</t>
         </is>
       </c>
-      <c r="E105" s="6" t="inlineStr">
+      <c r="E106" s="6" t="inlineStr">
         <is>
           <t>D001</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>Deliverys</t>
-        </is>
-      </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="inlineStr">
-        <is>
-          <t>Text (LABEL)</t>
-        </is>
-      </c>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>Nombre del repartidor</t>
-        </is>
-      </c>
-      <c r="E106" s="6" t="inlineStr">
-        <is>
-          <t>Juan Pérez</t>
         </is>
       </c>
     </row>
@@ -4889,22 +4948,22 @@
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Telefono</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>Nombre del repartidor</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>+56944444444</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
     </row>
@@ -4916,22 +4975,22 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Telefono</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
         <is>
-          <t>Correo con el que entra a la app (perfil Delivery)</t>
+          <t>Teléfono</t>
         </is>
       </c>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>juan.delivery@correo.com</t>
+          <t>+56944444444</t>
         </is>
       </c>
     </row>
@@ -4943,22 +5002,22 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Vehiculo</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Enum: Moto|Bicicleta|Auto|A pie</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Medio de transporte</t>
+          <t>Correo con el que entra a la app (perfil Delivery)</t>
         </is>
       </c>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>Moto</t>
+          <t>juan.delivery@correo.com</t>
         </is>
       </c>
     </row>
@@ -4970,22 +5029,22 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Patente</t>
+          <t>Vehiculo</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Moto|Bicicleta|Auto|A pie</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>Patente o placa</t>
+          <t>Medio de transporte</t>
         </is>
       </c>
       <c r="E110" s="6" t="inlineStr">
         <is>
-          <t>ABCD12</t>
+          <t>Moto</t>
         </is>
       </c>
     </row>
@@ -4997,22 +5056,22 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Patente</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Enum: Disponible|Ocupado|Inactivo</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Estado actual (cambia solo con automatización)</t>
+          <t>Patente o placa</t>
         </is>
       </c>
       <c r="E111" s="6" t="inlineStr">
         <is>
-          <t>Disponible</t>
+          <t>ABCD12</t>
         </is>
       </c>
     </row>
@@ -5024,22 +5083,22 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Tarifa_Base</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Enum: Disponible|Ocupado|Inactivo</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>Tarifa base por servicio</t>
+          <t>Estado actual (cambia solo con automatización)</t>
         </is>
       </c>
       <c r="E112" s="6" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5110,7 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Tarifa_Km</t>
+          <t>Tarifa_Base</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -5061,12 +5120,12 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Tarifa por km (opcional)</t>
+          <t>Tarifa base por servicio</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1000</t>
         </is>
       </c>
     </row>
@@ -5078,22 +5137,22 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Tarifa_Km</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>Yes/No</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Tarifa por km (opcional)</t>
         </is>
       </c>
       <c r="E114" s="6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>300</t>
         </is>
       </c>
     </row>
@@ -5105,22 +5164,22 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>Ultima_Ubicacion</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>Yes/No</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Última posición reportada</t>
+          <t>Habilitado</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
         <is>
-          <t>-33.4500,-70.6600</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5132,76 +5191,76 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
+          <t>Ultima_Ubicacion</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>LatLong</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>Última posición reportada</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t>-33.4500,-70.6600</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>Deliverys</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
           <t>Fecha_Ubicacion</t>
         </is>
       </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>Hora de la última posición</t>
         </is>
       </c>
-      <c r="E116" s="6" t="inlineStr">
+      <c r="E117" s="6" t="inlineStr">
         <is>
           <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="5" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
         <is>
           <t>Ventas</t>
         </is>
       </c>
-      <c r="B117" s="6" t="inlineStr">
+      <c r="B118" s="6" t="inlineStr">
         <is>
           <t>ID_Venta</t>
         </is>
       </c>
-      <c r="C117" s="6" t="inlineStr">
+      <c r="C118" s="6" t="inlineStr">
         <is>
           <t>Text (KEY)</t>
         </is>
       </c>
-      <c r="D117" s="6" t="inlineStr">
+      <c r="D118" s="6" t="inlineStr">
         <is>
           <t>Identificador. AppSheet: UNIQUEID() o correlativo</t>
         </is>
       </c>
-      <c r="E117" s="6" t="inlineStr">
+      <c r="E118" s="6" t="inlineStr">
         <is>
           <t>V000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="6" t="inlineStr">
-        <is>
-          <t>Ventas</t>
-        </is>
-      </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>Fecha_Hora</t>
-        </is>
-      </c>
-      <c r="C118" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>Automático: NOW()</t>
-        </is>
-      </c>
-      <c r="E118" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -5213,22 +5272,22 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>ID_Cliente</t>
+          <t>Fecha_Hora</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>Ref → Clientes</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Cliente (se puede crear desde la venta con Add new)</t>
+          <t>Automático: NOW()</t>
         </is>
       </c>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>CL0001</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -5240,22 +5299,22 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>Tipo_Entrega</t>
+          <t>ID_Cliente</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Enum: Retiro en local|Para servir|Delivery</t>
+          <t>Ref → Clientes</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>Si es Delivery se crea un servicio</t>
+          <t>Cliente (se puede crear desde la venta con Add new)</t>
         </is>
       </c>
       <c r="E120" s="6" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>CL0001</t>
         </is>
       </c>
     </row>
@@ -5267,22 +5326,22 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Tipo_Entrega</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Enum: Retiro en local|Para servir|Delivery</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Suma de Detalle_Venta (virtual column)</t>
+          <t>Si es Delivery se crea un servicio</t>
         </is>
       </c>
       <c r="E121" s="6" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>Delivery</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5353,7 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Subtotal</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -5304,12 +5363,12 @@
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>Descuento total</t>
+          <t>Suma de Detalle_Venta (virtual column)</t>
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3000</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5380,7 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>Costo_Delivery</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
@@ -5331,12 +5390,12 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Monto del delivery (si aplica)</t>
+          <t>Descuento total</t>
         </is>
       </c>
       <c r="E123" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5348,7 +5407,7 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Costo_Delivery</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
@@ -5358,12 +5417,12 @@
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>Subtotal - Descuento + Costo_Delivery (virtual)</t>
+          <t>Monto del delivery (si aplica)</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -5375,22 +5434,22 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>Metodo_Pago</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Enum: Efectivo|Tarjeta|Transferencia|Mixto</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>Forma de pago</t>
+          <t>Subtotal - Descuento + Costo_Delivery (virtual)</t>
         </is>
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>4500</t>
         </is>
       </c>
     </row>
@@ -5402,22 +5461,22 @@
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>Estado_Pago</t>
+          <t>Metodo_Pago</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>Enum: Pagado|Pendiente|Parcial</t>
+          <t>Enum: Efectivo|Tarjeta|Transferencia|Mixto</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
         <is>
-          <t>Estado del pago</t>
+          <t>Forma de pago</t>
         </is>
       </c>
       <c r="E126" s="6" t="inlineStr">
         <is>
-          <t>Pagado</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
@@ -5429,22 +5488,22 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Estado_Pago</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Enum: Borrador|Confirmada|En despacho|Entregada|Anulada</t>
+          <t>Enum: Pagado|Pendiente|Parcial</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>Estado de la venta</t>
+          <t>Estado del pago</t>
         </is>
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>Confirmada</t>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -5456,22 +5515,22 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>Tipo_Documento</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>Enum: Ticket|Boleta|Factura</t>
+          <t>Enum: Borrador|Confirmada|En despacho|Entregada|Anulada</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>Documento a emitir</t>
+          <t>Estado de la venta</t>
         </is>
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>Boleta</t>
+          <t>Confirmada</t>
         </is>
       </c>
     </row>
@@ -5483,22 +5542,22 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>Dia_Semana</t>
+          <t>Tipo_Documento</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Enum: Ticket|Boleta|Factura</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>Virtual/Apps Script: TEXT([Fecha_Hora],"dddd"). Sirve para KPI</t>
+          <t>Documento a emitir</t>
         </is>
       </c>
       <c r="E129" s="6" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>Boleta</t>
         </is>
       </c>
     </row>
@@ -5510,130 +5569,130 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
+          <t>Dia_Semana</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t>Virtual/Apps Script: TEXT([Fecha_Hora],"dddd"). Sirve para KPI</t>
+        </is>
+      </c>
+      <c r="E130" s="6" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
           <t>Usuario</t>
         </is>
       </c>
-      <c r="C130" s="6" t="inlineStr">
+      <c r="C131" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D130" s="6" t="inlineStr">
+      <c r="D131" s="6" t="inlineStr">
         <is>
           <t>Vendedor: USEREMAIL()</t>
         </is>
       </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="E131" s="6" t="inlineStr">
         <is>
           <t>ventas@minegocio.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="5" t="inlineStr">
-        <is>
-          <t>Detalle_Venta</t>
-        </is>
-      </c>
-      <c r="B131" s="6" t="inlineStr">
-        <is>
-          <t>ID_Detalle</t>
-        </is>
-      </c>
-      <c r="C131" s="6" t="inlineStr">
-        <is>
-          <t>Text (KEY)</t>
-        </is>
-      </c>
-      <c r="D131" s="6" t="inlineStr">
-        <is>
-          <t>Identificador</t>
-        </is>
-      </c>
-      <c r="E131" s="6" t="inlineStr">
-        <is>
-          <t>DV000001</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>Detalle_Venta</t>
+          <t>Ventas</t>
         </is>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>ID_Venta</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Ref → Ventas (Is a part of)</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>Venta a la que pertenece</t>
+          <t>Mesa, nombre o número para identificar el pedido en cocina</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>V000001</t>
+          <t>Mesa 4</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>Nota_Cocina</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>Indicación general para la cocina</t>
+        </is>
+      </c>
+      <c r="E133" s="6" t="inlineStr">
+        <is>
+          <t>Todo para llevar junto</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
           <t>Detalle_Venta</t>
         </is>
       </c>
-      <c r="B133" s="6" t="inlineStr">
-        <is>
-          <t>ID_Producto</t>
-        </is>
-      </c>
-      <c r="C133" s="6" t="inlineStr">
-        <is>
-          <t>Ref → Productos</t>
-        </is>
-      </c>
-      <c r="D133" s="6" t="inlineStr">
-        <is>
-          <t>Producto vendido</t>
-        </is>
-      </c>
-      <c r="E133" s="6" t="inlineStr">
-        <is>
-          <t>P0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="6" t="inlineStr">
-        <is>
-          <t>Detalle_Venta</t>
-        </is>
-      </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>Nombre_Producto</t>
+          <t>ID_Detalle</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>Copia del nombre al momento de vender (historial fiel)</t>
+          <t>Identificador</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>Bebida cola 1.5L</t>
+          <t>DV000001</t>
         </is>
       </c>
     </row>
@@ -5645,22 +5704,22 @@
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>ID_Categoria</t>
+          <t>ID_Venta</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Ref → Categorias</t>
+          <t>Ref → Ventas (Is a part of)</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Copia de categoría para KPI por categoría</t>
+          <t>Venta a la que pertenece</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -5672,22 +5731,22 @@
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>ID_Producto</t>
         </is>
       </c>
       <c r="C136" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Ref → Productos</t>
         </is>
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>Cantidad vendida</t>
+          <t>Producto vendido</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
@@ -5699,22 +5758,22 @@
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>Precio_Unitario</t>
+          <t>Nombre_Producto</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>Precio al momento de la venta</t>
+          <t>Copia del nombre al momento de vender (historial fiel)</t>
         </is>
       </c>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>Bebida cola 1.5L</t>
         </is>
       </c>
     </row>
@@ -5726,22 +5785,22 @@
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>Costo_Unitario</t>
+          <t>ID_Categoria</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Ref → Categorias</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>Costo al momento de la venta (para margen)</t>
+          <t>Copia de categoría para KPI por categoría</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>C001</t>
         </is>
       </c>
     </row>
@@ -5753,22 +5812,22 @@
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>Descuento de la línea</t>
+          <t>Cantidad vendida</t>
         </is>
       </c>
       <c r="E139" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5839,7 @@
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Precio_Unitario</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
@@ -5790,12 +5849,12 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>Cantidad × Precio - Descuento</t>
+          <t>Precio al momento de la venta</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -5807,115 +5866,115 @@
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Costo_Unitario</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>Fecha de la venta (para filtros y KPI)</t>
+          <t>Costo al momento de la venta (para margen)</t>
         </is>
       </c>
       <c r="E141" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026</t>
+          <t>900</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="5" t="inlineStr">
-        <is>
-          <t>Servicios_Delivery</t>
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>Detalle_Venta</t>
         </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
         <is>
-          <t>ID_Servicio</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
         <is>
-          <t>Text (KEY)</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D142" s="6" t="inlineStr">
         <is>
-          <t>Identificador</t>
+          <t>Descuento de la línea</t>
         </is>
       </c>
       <c r="E142" s="6" t="inlineStr">
         <is>
-          <t>S000001</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>Servicios_Delivery</t>
+          <t>Detalle_Venta</t>
         </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>ID_Venta</t>
+          <t>Subtotal</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>Ref → Ventas</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Venta asociada</t>
+          <t>Cantidad × Precio - Descuento</t>
         </is>
       </c>
       <c r="E143" s="6" t="inlineStr">
         <is>
-          <t>V000001</t>
+          <t>3000</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>Servicios_Delivery</t>
+          <t>Detalle_Venta</t>
         </is>
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>ID_Delivery</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C144" s="6" t="inlineStr">
         <is>
-          <t>Ref → Deliverys</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="D144" s="6" t="inlineStr">
         <is>
-          <t>Repartidor asignado</t>
+          <t>Fecha de la venta (para filtros y KPI)</t>
         </is>
       </c>
       <c r="E144" s="6" t="inlineStr">
         <is>
-          <t>D001</t>
+          <t>15-10-2026</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>Servicios_Delivery</t>
+          <t>Detalle_Venta</t>
         </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>Nombre_Delivery</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
@@ -5925,64 +5984,64 @@
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>Copia del nombre (historial fiel aunque cambie después)</t>
-        </is>
-      </c>
-      <c r="E145" s="6" t="inlineStr">
-        <is>
-          <t>Juan Pérez</t>
-        </is>
-      </c>
+          <t>Indicación para cocina de este producto (ej. sin cebolla)</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
+          <t>Detalle_Venta</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>Va_A_Cocina</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>Yes/No</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>Copia del producto: sale en la comanda</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
           <t>Servicios_Delivery</t>
         </is>
       </c>
-      <c r="B146" s="6" t="inlineStr">
-        <is>
-          <t>Fecha_Asignacion</t>
-        </is>
-      </c>
-      <c r="C146" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D146" s="6" t="inlineStr">
-        <is>
-          <t>Automático: NOW() al asignar</t>
-        </is>
-      </c>
-      <c r="E146" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="6" t="inlineStr">
-        <is>
-          <t>Servicios_Delivery</t>
-        </is>
-      </c>
       <c r="B147" s="6" t="inlineStr">
         <is>
-          <t>Fecha_Aceptado</t>
+          <t>ID_Servicio</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Se llena al presionar Aceptar</t>
-        </is>
-      </c>
-      <c r="E147" s="6" t="inlineStr"/>
+          <t>Identificador</t>
+        </is>
+      </c>
+      <c r="E147" s="6" t="inlineStr">
+        <is>
+          <t>S000001</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
@@ -5992,20 +6051,24 @@
       </c>
       <c r="B148" s="6" t="inlineStr">
         <is>
-          <t>Fecha_Finalizado</t>
+          <t>ID_Venta</t>
         </is>
       </c>
       <c r="C148" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Ref → Ventas</t>
         </is>
       </c>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t>Se llena al presionar Finalizar</t>
-        </is>
-      </c>
-      <c r="E148" s="6" t="inlineStr"/>
+          <t>Venta asociada</t>
+        </is>
+      </c>
+      <c r="E148" s="6" t="inlineStr">
+        <is>
+          <t>V000001</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
@@ -6015,22 +6078,22 @@
       </c>
       <c r="B149" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>ID_Delivery</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Ref → Deliverys</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Solo la fecha, para filtrar por rango</t>
+          <t>Repartidor asignado</t>
         </is>
       </c>
       <c r="E149" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026</t>
+          <t>D001</t>
         </is>
       </c>
     </row>
@@ -6042,22 +6105,22 @@
       </c>
       <c r="B150" s="6" t="inlineStr">
         <is>
-          <t>Direccion_Entrega</t>
+          <t>Nombre_Delivery</t>
         </is>
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>Dirección de destino</t>
+          <t>Copia del nombre (historial fiel aunque cambie después)</t>
         </is>
       </c>
       <c r="E150" s="6" t="inlineStr">
         <is>
-          <t>Av. Principal 123</t>
+          <t>Juan Pérez</t>
         </is>
       </c>
     </row>
@@ -6069,22 +6132,22 @@
       </c>
       <c r="B151" s="6" t="inlineStr">
         <is>
-          <t>Destino_LatLong</t>
+          <t>Fecha_Asignacion</t>
         </is>
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Coordenadas destino</t>
+          <t>Automático: NOW() al asignar</t>
         </is>
       </c>
       <c r="E151" s="6" t="inlineStr">
         <is>
-          <t>-33.4489,-70.6693</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
@@ -6096,24 +6159,20 @@
       </c>
       <c r="B152" s="6" t="inlineStr">
         <is>
-          <t>Origen_LatLong</t>
+          <t>Fecha_Aceptado</t>
         </is>
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t>Coordenadas del local</t>
-        </is>
-      </c>
-      <c r="E152" s="6" t="inlineStr">
-        <is>
-          <t>-33.4372,-70.6506</t>
-        </is>
-      </c>
+          <t>Se llena al presionar Aceptar</t>
+        </is>
+      </c>
+      <c r="E152" s="6" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
@@ -6123,24 +6182,20 @@
       </c>
       <c r="B153" s="6" t="inlineStr">
         <is>
-          <t>Distancia_Km</t>
+          <t>Fecha_Finalizado</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Km (manual o calculado con Apps Script/Maps)</t>
-        </is>
-      </c>
-      <c r="E153" s="6" t="inlineStr">
-        <is>
-          <t>4.2</t>
-        </is>
-      </c>
+          <t>Se llena al presionar Finalizar</t>
+        </is>
+      </c>
+      <c r="E153" s="6" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
@@ -6150,22 +6205,22 @@
       </c>
       <c r="B154" s="6" t="inlineStr">
         <is>
-          <t>Tiempo_Min</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="D154" s="6" t="inlineStr">
         <is>
-          <t>Duración en minutos</t>
+          <t>Solo la fecha, para filtrar por rango</t>
         </is>
       </c>
       <c r="E154" s="6" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15-10-2026</t>
         </is>
       </c>
     </row>
@@ -6177,22 +6232,22 @@
       </c>
       <c r="B155" s="6" t="inlineStr">
         <is>
-          <t>Monto_Delivery</t>
+          <t>Direccion_Entrega</t>
         </is>
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Costo del servicio</t>
+          <t>Dirección de destino</t>
         </is>
       </c>
       <c r="E155" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>Av. Principal 123</t>
         </is>
       </c>
     </row>
@@ -6204,22 +6259,22 @@
       </c>
       <c r="B156" s="6" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Destino_LatLong</t>
         </is>
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>Enum: Asignado|Aceptado|En camino|Finalizado|Rechazado|Cancelado</t>
+          <t>LatLong</t>
         </is>
       </c>
       <c r="D156" s="6" t="inlineStr">
         <is>
-          <t>Estado del servicio</t>
+          <t>Coordenadas destino</t>
         </is>
       </c>
       <c r="E156" s="6" t="inlineStr">
         <is>
-          <t>Asignado</t>
+          <t>-33.4489,-70.6693</t>
         </is>
       </c>
     </row>
@@ -6231,22 +6286,22 @@
       </c>
       <c r="B157" s="6" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Origen_LatLong</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>LongText</t>
+          <t>LatLong</t>
         </is>
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Instrucciones para el repartidor</t>
+          <t>Coordenadas del local</t>
         </is>
       </c>
       <c r="E157" s="6" t="inlineStr">
         <is>
-          <t>Llamar al llegar</t>
+          <t>-33.4372,-70.6506</t>
         </is>
       </c>
     </row>
@@ -6258,169 +6313,169 @@
       </c>
       <c r="B158" s="6" t="inlineStr">
         <is>
-          <t>Usuario_Asigna</t>
+          <t>Distancia_Km</t>
         </is>
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="D158" s="6" t="inlineStr">
         <is>
-          <t>Quién asignó</t>
+          <t>Km (manual o calculado con Apps Script/Maps)</t>
         </is>
       </c>
       <c r="E158" s="6" t="inlineStr">
         <is>
-          <t>ventas@minegocio.com</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="5" t="inlineStr">
-        <is>
-          <t>Ubicaciones_Delivery</t>
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>Servicios_Delivery</t>
         </is>
       </c>
       <c r="B159" s="6" t="inlineStr">
         <is>
-          <t>ID_Ubic</t>
+          <t>Tiempo_Min</t>
         </is>
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Text (KEY)</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>Identificador</t>
+          <t>Duración en minutos</t>
         </is>
       </c>
       <c r="E159" s="6" t="inlineStr">
         <is>
-          <t>UB000001</t>
+          <t>18</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="6" t="inlineStr">
         <is>
-          <t>Ubicaciones_Delivery</t>
+          <t>Servicios_Delivery</t>
         </is>
       </c>
       <c r="B160" s="6" t="inlineStr">
         <is>
-          <t>ID_Servicio</t>
+          <t>Monto_Delivery</t>
         </is>
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>Ref → Servicios_Delivery</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D160" s="6" t="inlineStr">
         <is>
-          <t>Servicio en curso</t>
+          <t>Costo del servicio</t>
         </is>
       </c>
       <c r="E160" s="6" t="inlineStr">
         <is>
-          <t>S000001</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>Ubicaciones_Delivery</t>
+          <t>Servicios_Delivery</t>
         </is>
       </c>
       <c r="B161" s="6" t="inlineStr">
         <is>
-          <t>ID_Delivery</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Ref → Deliverys</t>
+          <t>Enum: Asignado|Aceptado|En camino|Finalizado|Rechazado|Cancelado</t>
         </is>
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Repartidor</t>
+          <t>Estado del servicio</t>
         </is>
       </c>
       <c r="E161" s="6" t="inlineStr">
         <is>
-          <t>D001</t>
+          <t>Asignado</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>Ubicaciones_Delivery</t>
+          <t>Servicios_Delivery</t>
         </is>
       </c>
       <c r="B162" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>Notas</t>
         </is>
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>LatLong</t>
+          <t>LongText</t>
         </is>
       </c>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t>Posición registrada (AppSheet: HERE())</t>
+          <t>Instrucciones para el repartidor</t>
         </is>
       </c>
       <c r="E162" s="6" t="inlineStr">
         <is>
-          <t>-33.4470,-70.6620</t>
+          <t>Llamar al llegar</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>Ubicaciones_Delivery</t>
+          <t>Servicios_Delivery</t>
         </is>
       </c>
       <c r="B163" s="6" t="inlineStr">
         <is>
-          <t>Fecha_Hora</t>
+          <t>Usuario_Asigna</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Momento del registro</t>
+          <t>Quién asignó</t>
         </is>
       </c>
       <c r="E163" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>ventas@minegocio.com</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="5" t="inlineStr">
         <is>
-          <t>Documentos</t>
+          <t>Ubicaciones_Delivery</t>
         </is>
       </c>
       <c r="B164" s="6" t="inlineStr">
         <is>
-          <t>ID_Documento</t>
+          <t>ID_Ubic</t>
         </is>
       </c>
       <c r="C164" s="6" t="inlineStr">
@@ -6435,142 +6490,142 @@
       </c>
       <c r="E164" s="6" t="inlineStr">
         <is>
-          <t>DOC0001</t>
+          <t>UB000001</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>Documentos</t>
+          <t>Ubicaciones_Delivery</t>
         </is>
       </c>
       <c r="B165" s="6" t="inlineStr">
         <is>
-          <t>ID_Venta</t>
+          <t>ID_Servicio</t>
         </is>
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Ref → Ventas</t>
+          <t>Ref → Servicios_Delivery</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Venta origen</t>
+          <t>Servicio en curso</t>
         </is>
       </c>
       <c r="E165" s="6" t="inlineStr">
         <is>
-          <t>V000001</t>
+          <t>S000001</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="6" t="inlineStr">
         <is>
-          <t>Documentos</t>
+          <t>Ubicaciones_Delivery</t>
         </is>
       </c>
       <c r="B166" s="6" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>ID_Delivery</t>
         </is>
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Enum: Ticket|Boleta|Factura</t>
+          <t>Ref → Deliverys</t>
         </is>
       </c>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t>Tipo de documento</t>
+          <t>Repartidor</t>
         </is>
       </c>
       <c r="E166" s="6" t="inlineStr">
         <is>
-          <t>Boleta</t>
+          <t>D001</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>Documentos</t>
+          <t>Ubicaciones_Delivery</t>
         </is>
       </c>
       <c r="B167" s="6" t="inlineStr">
         <is>
-          <t>Folio</t>
+          <t>LatLong</t>
         </is>
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>LatLong</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Número correlativo interno (o folio SII si usas facturación electrónica)</t>
+          <t>Posición registrada (AppSheet: HERE())</t>
         </is>
       </c>
       <c r="E167" s="6" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>-33.4470,-70.6620</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="6" t="inlineStr">
         <is>
+          <t>Ubicaciones_Delivery</t>
+        </is>
+      </c>
+      <c r="B168" s="6" t="inlineStr">
+        <is>
+          <t>Fecha_Hora</t>
+        </is>
+      </c>
+      <c r="C168" s="6" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="D168" s="6" t="inlineStr">
+        <is>
+          <t>Momento del registro</t>
+        </is>
+      </c>
+      <c r="E168" s="6" t="inlineStr">
+        <is>
+          <t>15-10-2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
           <t>Documentos</t>
         </is>
       </c>
-      <c r="B168" s="6" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C168" s="6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="D168" s="6" t="inlineStr">
-        <is>
-          <t>Emisión</t>
-        </is>
-      </c>
-      <c r="E168" s="6" t="inlineStr">
-        <is>
-          <t>15-10-2026 12:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="6" t="inlineStr">
-        <is>
-          <t>Documentos</t>
-        </is>
-      </c>
       <c r="B169" s="6" t="inlineStr">
         <is>
-          <t>Neto</t>
+          <t>ID_Documento</t>
         </is>
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Monto neto</t>
+          <t>Identificador</t>
         </is>
       </c>
       <c r="E169" s="6" t="inlineStr">
         <is>
-          <t>3782</t>
+          <t>DOC0001</t>
         </is>
       </c>
     </row>
@@ -6582,22 +6637,22 @@
       </c>
       <c r="B170" s="6" t="inlineStr">
         <is>
-          <t>Impuesto</t>
+          <t>ID_Venta</t>
         </is>
       </c>
       <c r="C170" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Ref → Ventas</t>
         </is>
       </c>
       <c r="D170" s="6" t="inlineStr">
         <is>
-          <t>IVA u otro impuesto</t>
+          <t>Venta origen</t>
         </is>
       </c>
       <c r="E170" s="6" t="inlineStr">
         <is>
-          <t>718</t>
+          <t>V000001</t>
         </is>
       </c>
     </row>
@@ -6609,22 +6664,22 @@
       </c>
       <c r="B171" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Enum: Ticket|Boleta|Factura</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Tipo de documento</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>Boleta</t>
         </is>
       </c>
     </row>
@@ -6636,22 +6691,22 @@
       </c>
       <c r="B172" s="6" t="inlineStr">
         <is>
-          <t>Formato</t>
+          <t>Folio</t>
         </is>
       </c>
       <c r="C172" s="6" t="inlineStr">
         <is>
-          <t>Enum: Termica 58mm|Termica 80mm|A4 Carta</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D172" s="6" t="inlineStr">
         <is>
-          <t>Formato de impresión</t>
+          <t>Número correlativo interno (o folio SII si usas facturación electrónica)</t>
         </is>
       </c>
       <c r="E172" s="6" t="inlineStr">
         <is>
-          <t>Termica 80mm</t>
+          <t>1001</t>
         </is>
       </c>
     </row>
@@ -6663,160 +6718,160 @@
       </c>
       <c r="B173" s="6" t="inlineStr">
         <is>
-          <t>PDF_URL</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>PDF generado por Apps Script en Drive</t>
-        </is>
-      </c>
-      <c r="E173" s="6" t="inlineStr"/>
+          <t>Emisión</t>
+        </is>
+      </c>
+      <c r="E173" s="6" t="inlineStr">
+        <is>
+          <t>15-10-2026 12:30</t>
+        </is>
+      </c>
     </row>
     <row r="174">
-      <c r="A174" s="5" t="inlineStr">
-        <is>
-          <t>Categorias_Conocimiento</t>
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>Documentos</t>
         </is>
       </c>
       <c r="B174" s="6" t="inlineStr">
         <is>
-          <t>ID_CatCon</t>
+          <t>Neto</t>
         </is>
       </c>
       <c r="C174" s="6" t="inlineStr">
         <is>
-          <t>Text (KEY)</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D174" s="6" t="inlineStr">
         <is>
-          <t>Identificador</t>
+          <t>Monto neto</t>
         </is>
       </c>
       <c r="E174" s="6" t="inlineStr">
         <is>
-          <t>CK01</t>
+          <t>3782</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="6" t="inlineStr">
         <is>
-          <t>Categorias_Conocimiento</t>
+          <t>Documentos</t>
         </is>
       </c>
       <c r="B175" s="6" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Impuesto</t>
         </is>
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>Text (LABEL)</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Nombre de la categoría</t>
+          <t>IVA u otro impuesto</t>
         </is>
       </c>
       <c r="E175" s="6" t="inlineStr">
         <is>
-          <t>Recetas</t>
+          <t>718</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="6" t="inlineStr">
         <is>
-          <t>Categorias_Conocimiento</t>
+          <t>Documentos</t>
         </is>
       </c>
       <c r="B176" s="6" t="inlineStr">
         <is>
-          <t>Imagen</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="C176" s="6" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D176" s="6" t="inlineStr">
         <is>
-          <t>Imagen opcional</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E176" s="6" t="inlineStr">
         <is>
-          <t>Conocimiento_Images/recetas.png</t>
+          <t>4500</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="5" t="inlineStr">
-        <is>
-          <t>Conocimiento</t>
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>Documentos</t>
         </is>
       </c>
       <c r="B177" s="6" t="inlineStr">
         <is>
-          <t>ID_Conocimiento</t>
+          <t>Formato</t>
         </is>
       </c>
       <c r="C177" s="6" t="inlineStr">
         <is>
-          <t>Text (KEY)</t>
+          <t>Enum: Termica 58mm|Termica 80mm|A4 Carta</t>
         </is>
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>Identificador</t>
+          <t>Formato de impresión</t>
         </is>
       </c>
       <c r="E177" s="6" t="inlineStr">
         <is>
-          <t>K0001</t>
+          <t>Termica 80mm</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="6" t="inlineStr">
         <is>
-          <t>Conocimiento</t>
+          <t>Documentos</t>
         </is>
       </c>
       <c r="B178" s="6" t="inlineStr">
         <is>
-          <t>Titulo</t>
+          <t>PDF_URL</t>
         </is>
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>Text (LABEL)</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t>Título del documento</t>
-        </is>
-      </c>
-      <c r="E178" s="6" t="inlineStr">
-        <is>
-          <t>Preparación salsa base</t>
-        </is>
-      </c>
+          <t>PDF generado por Apps Script en Drive</t>
+        </is>
+      </c>
+      <c r="E178" s="6" t="inlineStr"/>
     </row>
     <row r="179">
-      <c r="A179" s="6" t="inlineStr">
-        <is>
-          <t>Conocimiento</t>
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>Categorias_Conocimiento</t>
         </is>
       </c>
       <c r="B179" s="6" t="inlineStr">
@@ -6826,12 +6881,12 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>Ref → Categorias_Conocimiento</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>Categoría</t>
+          <t>Identificador</t>
         </is>
       </c>
       <c r="E179" s="6" t="inlineStr">
@@ -6843,81 +6898,81 @@
     <row r="180">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>Conocimiento</t>
+          <t>Categorias_Conocimiento</t>
         </is>
       </c>
       <c r="B180" s="6" t="inlineStr">
         <is>
-          <t>Archivo_PDF</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D180" s="6" t="inlineStr">
         <is>
-          <t>PDF subido (se guarda en Drive)</t>
+          <t>Nombre de la categoría</t>
         </is>
       </c>
       <c r="E180" s="6" t="inlineStr">
         <is>
-          <t>Conocimiento_Files/salsa_base.pdf</t>
+          <t>Recetas</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
+          <t>Categorias_Conocimiento</t>
+        </is>
+      </c>
+      <c r="B181" s="6" t="inlineStr">
+        <is>
+          <t>Imagen</t>
+        </is>
+      </c>
+      <c r="C181" s="6" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D181" s="6" t="inlineStr">
+        <is>
+          <t>Imagen opcional</t>
+        </is>
+      </c>
+      <c r="E181" s="6" t="inlineStr">
+        <is>
+          <t>Conocimiento_Images/recetas.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
           <t>Conocimiento</t>
         </is>
       </c>
-      <c r="B181" s="6" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="C181" s="6" t="inlineStr">
-        <is>
-          <t>LongText</t>
-        </is>
-      </c>
-      <c r="D181" s="6" t="inlineStr">
-        <is>
-          <t>Resumen</t>
-        </is>
-      </c>
-      <c r="E181" s="6" t="inlineStr">
-        <is>
-          <t>Receta estándar de salsa base</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="6" t="inlineStr">
-        <is>
-          <t>Conocimiento</t>
-        </is>
-      </c>
       <c r="B182" s="6" t="inlineStr">
         <is>
-          <t>Etiquetas</t>
+          <t>ID_Conocimiento</t>
         </is>
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>EnumList (Allow other values)</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t>Etiquetas para buscar</t>
+          <t>Identificador</t>
         </is>
       </c>
       <c r="E182" s="6" t="inlineStr">
         <is>
-          <t>salsa, base</t>
+          <t>K0001</t>
         </is>
       </c>
     </row>
@@ -6929,22 +6984,22 @@
       </c>
       <c r="B183" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Titulo</t>
         </is>
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Text (LABEL)</t>
         </is>
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Automático</t>
+          <t>Título del documento</t>
         </is>
       </c>
       <c r="E183" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>Preparación salsa base</t>
         </is>
       </c>
     </row>
@@ -6956,184 +7011,184 @@
       </c>
       <c r="B184" s="6" t="inlineStr">
         <is>
-          <t>Usuario</t>
+          <t>ID_CatCon</t>
         </is>
       </c>
       <c r="C184" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Ref → Categorias_Conocimiento</t>
         </is>
       </c>
       <c r="D184" s="6" t="inlineStr">
         <is>
-          <t>Quién lo subió</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="E184" s="6" t="inlineStr">
         <is>
-          <t>master@minegocio.com</t>
+          <t>CK01</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="5" t="inlineStr">
-        <is>
-          <t>Alertas</t>
+      <c r="A185" s="6" t="inlineStr">
+        <is>
+          <t>Conocimiento</t>
         </is>
       </c>
       <c r="B185" s="6" t="inlineStr">
         <is>
-          <t>ID_Alerta</t>
+          <t>Archivo_PDF</t>
         </is>
       </c>
       <c r="C185" s="6" t="inlineStr">
         <is>
-          <t>Text (KEY)</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>Identificador</t>
+          <t>PDF subido (se guarda en Drive)</t>
         </is>
       </c>
       <c r="E185" s="6" t="inlineStr">
         <is>
-          <t>A000001</t>
+          <t>Conocimiento_Files/salsa_base.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="6" t="inlineStr">
         <is>
-          <t>Alertas</t>
+          <t>Conocimiento</t>
         </is>
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Descripcion</t>
         </is>
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>LongText</t>
         </is>
       </c>
       <c r="D186" s="6" t="inlineStr">
         <is>
-          <t>Automático</t>
+          <t>Resumen</t>
         </is>
       </c>
       <c r="E186" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>Receta estándar de salsa base</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="6" t="inlineStr">
         <is>
-          <t>Alertas</t>
+          <t>Conocimiento</t>
         </is>
       </c>
       <c r="B187" s="6" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Etiquetas</t>
         </is>
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>Enum: Stock minimo|Delivery finalizado|Delivery rechazado|Otro</t>
+          <t>EnumList (Allow other values)</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Tipo de alerta</t>
+          <t>Etiquetas para buscar</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
         <is>
-          <t>Stock minimo</t>
+          <t>salsa, base</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="6" t="inlineStr">
         <is>
-          <t>Alertas</t>
+          <t>Conocimiento</t>
         </is>
       </c>
       <c r="B188" s="6" t="inlineStr">
         <is>
-          <t>Referencia</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D188" s="6" t="inlineStr">
         <is>
-          <t>ID_Producto o ID_Servicio</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="E188" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
+          <t>Conocimiento</t>
+        </is>
+      </c>
+      <c r="B189" s="6" t="inlineStr">
+        <is>
+          <t>Usuario</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D189" s="6" t="inlineStr">
+        <is>
+          <t>Quién lo subió</t>
+        </is>
+      </c>
+      <c r="E189" s="6" t="inlineStr">
+        <is>
+          <t>master@minegocio.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="inlineStr">
+        <is>
           <t>Alertas</t>
         </is>
       </c>
-      <c r="B189" s="6" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="C189" s="6" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="D189" s="6" t="inlineStr">
-        <is>
-          <t>Texto de la alerta</t>
-        </is>
-      </c>
-      <c r="E189" s="6" t="inlineStr">
-        <is>
-          <t>Bebida cola 1.5L llegó al stock mínimo (10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="6" t="inlineStr">
-        <is>
-          <t>Alertas</t>
-        </is>
-      </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
-          <t>Para_Rol</t>
+          <t>ID_Alerta</t>
         </is>
       </c>
       <c r="C190" s="6" t="inlineStr">
         <is>
-          <t>Ref → Roles</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D190" s="6" t="inlineStr">
         <is>
-          <t>Rol que debe verla</t>
+          <t>Identificador</t>
         </is>
       </c>
       <c r="E190" s="6" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>A000001</t>
         </is>
       </c>
     </row>
@@ -7145,184 +7200,184 @@
       </c>
       <c r="B191" s="6" t="inlineStr">
         <is>
-          <t>Leida</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>Yes/No</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Marcada como leída</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="E191" s="6" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>15-10-2026 12:30</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="5" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
+      <c r="A192" s="6" t="inlineStr">
+        <is>
+          <t>Alertas</t>
         </is>
       </c>
       <c r="B192" s="6" t="inlineStr">
         <is>
-          <t>ID_Log</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C192" s="6" t="inlineStr">
         <is>
-          <t>Text (KEY)</t>
+          <t>Enum: Stock minimo|Delivery finalizado|Delivery rechazado|Otro</t>
         </is>
       </c>
       <c r="D192" s="6" t="inlineStr">
         <is>
-          <t>Identificador</t>
+          <t>Tipo de alerta</t>
         </is>
       </c>
       <c r="E192" s="6" t="inlineStr">
         <is>
-          <t>L000001</t>
+          <t>Stock minimo</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Alertas</t>
         </is>
       </c>
       <c r="B193" s="6" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Automático</t>
+          <t>ID_Producto o ID_Servicio</t>
         </is>
       </c>
       <c r="E193" s="6" t="inlineStr">
         <is>
-          <t>15-10-2026 12:30</t>
+          <t>P0001</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="6" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Alertas</t>
         </is>
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t>Usuario</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D194" s="6" t="inlineStr">
         <is>
-          <t>Quién</t>
+          <t>Texto de la alerta</t>
         </is>
       </c>
       <c r="E194" s="6" t="inlineStr">
         <is>
-          <t>master@minegocio.com</t>
+          <t>Bebida cola 1.5L llegó al stock mínimo (10)</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Alertas</t>
         </is>
       </c>
       <c r="B195" s="6" t="inlineStr">
         <is>
-          <t>Modulo</t>
+          <t>Para_Rol</t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Ref → Roles</t>
         </is>
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Módulo afectado</t>
+          <t>Rol que debe verla</t>
         </is>
       </c>
       <c r="E195" s="6" t="inlineStr">
         <is>
-          <t>Inventario</t>
+          <t>R01</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="6" t="inlineStr">
         <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="B196" s="6" t="inlineStr">
+        <is>
+          <t>Leida</t>
+        </is>
+      </c>
+      <c r="C196" s="6" t="inlineStr">
+        <is>
+          <t>Yes/No</t>
+        </is>
+      </c>
+      <c r="D196" s="6" t="inlineStr">
+        <is>
+          <t>Marcada como leída</t>
+        </is>
+      </c>
+      <c r="E196" s="6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="inlineStr">
+        <is>
           <t>Auditoria</t>
         </is>
       </c>
-      <c r="B196" s="6" t="inlineStr">
-        <is>
-          <t>Accion</t>
-        </is>
-      </c>
-      <c r="C196" s="6" t="inlineStr">
-        <is>
-          <t>Enum: Crear|Editar|Eliminar|Exportar|Login</t>
-        </is>
-      </c>
-      <c r="D196" s="6" t="inlineStr">
-        <is>
-          <t>Qué hizo</t>
-        </is>
-      </c>
-      <c r="E196" s="6" t="inlineStr">
-        <is>
-          <t>Crear</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" s="6" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>Registro</t>
+          <t>ID_Log</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Text (KEY)</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>ID del registro afectado</t>
+          <t>Identificador</t>
         </is>
       </c>
       <c r="E197" s="6" t="inlineStr">
         <is>
-          <t>P0001</t>
+          <t>L000001</t>
         </is>
       </c>
     </row>
@@ -7334,27 +7389,162 @@
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C198" s="6" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="D198" s="6" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="E198" s="6" t="inlineStr">
+        <is>
+          <t>15-10-2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="6" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>Usuario</t>
+        </is>
+      </c>
+      <c r="C199" s="6" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>Quién</t>
+        </is>
+      </c>
+      <c r="E199" s="6" t="inlineStr">
+        <is>
+          <t>master@minegocio.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="6" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="B200" s="6" t="inlineStr">
+        <is>
+          <t>Modulo</t>
+        </is>
+      </c>
+      <c r="C200" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D200" s="6" t="inlineStr">
+        <is>
+          <t>Módulo afectado</t>
+        </is>
+      </c>
+      <c r="E200" s="6" t="inlineStr">
+        <is>
+          <t>Inventario</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="6" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="B201" s="6" t="inlineStr">
+        <is>
+          <t>Accion</t>
+        </is>
+      </c>
+      <c r="C201" s="6" t="inlineStr">
+        <is>
+          <t>Enum: Crear|Editar|Eliminar|Exportar|Login</t>
+        </is>
+      </c>
+      <c r="D201" s="6" t="inlineStr">
+        <is>
+          <t>Qué hizo</t>
+        </is>
+      </c>
+      <c r="E201" s="6" t="inlineStr">
+        <is>
+          <t>Crear</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="6" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="B202" s="6" t="inlineStr">
+        <is>
+          <t>Registro</t>
+        </is>
+      </c>
+      <c r="C202" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D202" s="6" t="inlineStr">
+        <is>
+          <t>ID del registro afectado</t>
+        </is>
+      </c>
+      <c r="E202" s="6" t="inlineStr">
+        <is>
+          <t>P0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="6" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="B203" s="6" t="inlineStr">
+        <is>
           <t>Detalle</t>
         </is>
       </c>
-      <c r="C198" s="6" t="inlineStr">
+      <c r="C203" s="6" t="inlineStr">
         <is>
           <t>LongText</t>
         </is>
       </c>
-      <c r="D198" s="6" t="inlineStr">
+      <c r="D203" s="6" t="inlineStr">
         <is>
           <t>Detalle del cambio</t>
         </is>
       </c>
-      <c r="E198" s="6" t="inlineStr">
+      <c r="E203" s="6" t="inlineStr">
         <is>
           <t>Producto creado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E198"/>
+  <autoFilter ref="A1:E203"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9713,7 +9903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9877,45 +10067,79 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>ORIGEN_LATLONG</t>
+          <t>FORMATO_COMANDA</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>-33.4372,-70.6506</t>
+          <t>Termica 80mm</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Coordenadas del local</t>
+          <t>Formato del ticket de cocina</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>ALERTA_STOCK_ACTIVA</t>
+          <t>COMANDA_AUTO</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Activa las alertas de stock mínimo</t>
+          <t>TRUE = al vender se abre sola la impresión de la comanda</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
+          <t>ORIGEN_LATLONG</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>-33.4372,-70.6506</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Coordenadas del local</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>ALERTA_STOCK_ACTIVA</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Activa las alertas de stock mínimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
           <t>LOGO</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr"/>
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>URL del logo (se sube desde Configuración)</t>
         </is>

</xml_diff>